<commit_message>
Main changes according to comments recieved
</commit_message>
<xml_diff>
--- a/predicted_pumps_all_params.xlsx
+++ b/predicted_pumps_all_params.xlsx
@@ -472,34 +472,34 @@
         <v>46023</v>
       </c>
       <c r="C2">
-        <v>58.03540324927923</v>
+        <v>59.0529130692578</v>
       </c>
       <c r="D2">
-        <v>232.2044316394805</v>
+        <v>232.4813234385547</v>
       </c>
       <c r="E2">
-        <v>36.31127839831927</v>
+        <v>36.77861414301218</v>
       </c>
       <c r="F2">
-        <v>0.6260696107911041</v>
+        <v>0.6292510957748514</v>
       </c>
       <c r="G2">
-        <v>41.62777349355333</v>
+        <v>43.35861622014306</v>
       </c>
       <c r="H2">
-        <v>10569.74260763795</v>
+        <v>10570.89891657605</v>
       </c>
       <c r="I2">
-        <v>198.9545863920108</v>
+        <v>198.9115862938901</v>
       </c>
       <c r="J2">
-        <v>49.79177015081155</v>
+        <v>49.79279388863253</v>
       </c>
       <c r="K2">
-        <v>86.61975108136255</v>
+        <v>86.9508008372468</v>
       </c>
       <c r="L2">
-        <v>0.1916639540570069</v>
+        <v>0.1845654956327074</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -510,34 +510,34 @@
         <v>46054</v>
       </c>
       <c r="C3">
-        <v>58.07940918637959</v>
+        <v>67.10794872022655</v>
       </c>
       <c r="D3">
-        <v>232.4655268066129</v>
+        <v>232.1406940518652</v>
       </c>
       <c r="E3">
-        <v>36.9944556177124</v>
+        <v>36.8985608476813</v>
       </c>
       <c r="F3">
-        <v>0.632484829672328</v>
+        <v>0.6276776423201323</v>
       </c>
       <c r="G3">
-        <v>41.67504702496781</v>
+        <v>42.14714819641715</v>
       </c>
       <c r="H3">
-        <v>10570.96487710055</v>
+        <v>10574.65367567577</v>
       </c>
       <c r="I3">
-        <v>198.8287589023937</v>
+        <v>198.9066963376182</v>
       </c>
       <c r="J3">
-        <v>49.7926639909068</v>
+        <v>49.79253380795006</v>
       </c>
       <c r="K3">
-        <v>86.93984167360941</v>
+        <v>86.95201309295845</v>
       </c>
       <c r="L3">
-        <v>0.1998253448687207</v>
+        <v>0.1645820728678055</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -548,34 +548,34 @@
         <v>46082</v>
       </c>
       <c r="C4">
-        <v>58.03400429925554</v>
+        <v>55.94851147068171</v>
       </c>
       <c r="D4">
-        <v>232.4795360150252</v>
+        <v>232.4545232957115</v>
       </c>
       <c r="E4">
-        <v>36.75009771148944</v>
+        <v>36.3774548177147</v>
       </c>
       <c r="F4">
-        <v>0.644438850539004</v>
+        <v>0.6243729220156651</v>
       </c>
       <c r="G4">
-        <v>41.6026094762909</v>
+        <v>47.31174631723967</v>
       </c>
       <c r="H4">
-        <v>10575.14282097592</v>
+        <v>10575.57660634176</v>
       </c>
       <c r="I4">
-        <v>199.0016421469733</v>
+        <v>198.9975489641181</v>
       </c>
       <c r="J4">
-        <v>49.79263351163569</v>
+        <v>49.79220459858759</v>
       </c>
       <c r="K4">
-        <v>86.8796805450107</v>
+        <v>87.04275712026583</v>
       </c>
       <c r="L4">
-        <v>0.189890659865144</v>
+        <v>0.1556081796661224</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -586,34 +586,34 @@
         <v>46113</v>
       </c>
       <c r="C5">
-        <v>58.11714680133749</v>
+        <v>58.41976563745753</v>
       </c>
       <c r="D5">
-        <v>232.4792630824179</v>
+        <v>232.1365082772284</v>
       </c>
       <c r="E5">
-        <v>37.06727867736715</v>
+        <v>36.8003170189853</v>
       </c>
       <c r="F5">
-        <v>0.6258491118961487</v>
+        <v>0.6455656745063029</v>
       </c>
       <c r="G5">
-        <v>41.90890505659013</v>
+        <v>35</v>
       </c>
       <c r="H5">
-        <v>10569.96073086656</v>
+        <v>10574.09125699381</v>
       </c>
       <c r="I5">
-        <v>198.8427076850793</v>
+        <v>198.8176898379818</v>
       </c>
       <c r="J5">
-        <v>49.79264988002596</v>
+        <v>49.79228894739577</v>
       </c>
       <c r="K5">
-        <v>86.98606708943346</v>
+        <v>86.9565383573327</v>
       </c>
       <c r="L5">
-        <v>0.1989745756919757</v>
+        <v>0.1770222220535517</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -624,34 +624,34 @@
         <v>46143</v>
       </c>
       <c r="C6">
-        <v>58.03435632120549</v>
+        <v>56.80755418236129</v>
       </c>
       <c r="D6">
-        <v>232.1443641660832</v>
+        <v>232.4694027777863</v>
       </c>
       <c r="E6">
-        <v>36.33862348701887</v>
+        <v>37.44715967403928</v>
       </c>
       <c r="F6">
-        <v>0.6275478189441117</v>
+        <v>0.6429282318018598</v>
       </c>
       <c r="G6">
-        <v>41.93593326369341</v>
+        <v>35</v>
       </c>
       <c r="H6">
-        <v>10569.68357492155</v>
+        <v>10570.72714494708</v>
       </c>
       <c r="I6">
-        <v>198.7670057547843</v>
+        <v>198.8060129299708</v>
       </c>
       <c r="J6">
-        <v>49.79185906293075</v>
+        <v>49.7926706917462</v>
       </c>
       <c r="K6">
-        <v>86.68421720483546</v>
+        <v>86.92411979892606</v>
       </c>
       <c r="L6">
-        <v>0.1930460520475361</v>
+        <v>0.1754359313628572</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -662,34 +662,34 @@
         <v>46174</v>
       </c>
       <c r="C7">
-        <v>58.03470771383116</v>
+        <v>55.18172222608885</v>
       </c>
       <c r="D7">
-        <v>232.4501534426467</v>
+        <v>232.455246323853</v>
       </c>
       <c r="E7">
-        <v>37.10279903669802</v>
+        <v>36.50818336915118</v>
       </c>
       <c r="F7">
-        <v>0.6440689108532547</v>
+        <v>0.6276803000857575</v>
       </c>
       <c r="G7">
-        <v>41.67821526797594</v>
+        <v>35</v>
       </c>
       <c r="H7">
-        <v>10575.64527028684</v>
+        <v>10574.75004242173</v>
       </c>
       <c r="I7">
-        <v>198.8324181133966</v>
+        <v>198.6507911541939</v>
       </c>
       <c r="J7">
-        <v>49.79210480008093</v>
+        <v>49.7924129134165</v>
       </c>
       <c r="K7">
-        <v>86.72437863338146</v>
+        <v>86.64332730940419</v>
       </c>
       <c r="L7">
-        <v>0.1877163353139346</v>
+        <v>0.1643374421804706</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -700,34 +700,34 @@
         <v>46204</v>
       </c>
       <c r="C8">
-        <v>58.03383524341542</v>
+        <v>59.38521977787985</v>
       </c>
       <c r="D8">
-        <v>232.4792193120792</v>
+        <v>232.1353465310991</v>
       </c>
       <c r="E8">
-        <v>36.38214074017905</v>
+        <v>36.50651908819582</v>
       </c>
       <c r="F8">
-        <v>0.6342197783409631</v>
+        <v>0.6231241872338341</v>
       </c>
       <c r="G8">
-        <v>41.9311116088302</v>
+        <v>50.65209082397802</v>
       </c>
       <c r="H8">
-        <v>10575.6426409021</v>
+        <v>10573.88450436656</v>
       </c>
       <c r="I8">
-        <v>198.775081598887</v>
+        <v>198.9181486027678</v>
       </c>
       <c r="J8">
-        <v>49.79270467955816</v>
+        <v>49.79241736345458</v>
       </c>
       <c r="K8">
-        <v>86.8465960902317</v>
+        <v>87.02597874721422</v>
       </c>
       <c r="L8">
-        <v>0.187788921281154</v>
+        <v>0.1575181705407147</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -738,34 +738,34 @@
         <v>46235</v>
       </c>
       <c r="C9">
-        <v>58.03428522907227</v>
+        <v>56.00475078349994</v>
       </c>
       <c r="D9">
-        <v>232.1446857585663</v>
+        <v>232.4809856998034</v>
       </c>
       <c r="E9">
-        <v>36.78636074780204</v>
+        <v>36.22215377174762</v>
       </c>
       <c r="F9">
-        <v>0.6369675344776595</v>
+        <v>0.6357828215187324</v>
       </c>
       <c r="G9">
-        <v>41.65807621118233</v>
+        <v>61.4700015259759</v>
       </c>
       <c r="H9">
-        <v>10570.01830981972</v>
+        <v>10570.40996128002</v>
       </c>
       <c r="I9">
-        <v>198.7846516857069</v>
+        <v>198.8993331103836</v>
       </c>
       <c r="J9">
-        <v>49.79241590493317</v>
+        <v>49.79263094512986</v>
       </c>
       <c r="K9">
-        <v>86.84574370830461</v>
+        <v>86.79896635594027</v>
       </c>
       <c r="L9">
-        <v>0.1942518834060525</v>
+        <v>0.1535273700589067</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -776,34 +776,34 @@
         <v>46266</v>
       </c>
       <c r="C10">
-        <v>58.11609417808965</v>
+        <v>78.40298842050335</v>
       </c>
       <c r="D10">
-        <v>232.1464987300243</v>
+        <v>232.4678975364058</v>
       </c>
       <c r="E10">
-        <v>36.40168844247169</v>
+        <v>37.37543122579712</v>
       </c>
       <c r="F10">
-        <v>0.6288844190222719</v>
+        <v>0.6268415522457054</v>
       </c>
       <c r="G10">
-        <v>41.62105277583212</v>
+        <v>47.08443925014418</v>
       </c>
       <c r="H10">
-        <v>10573.9303127834</v>
+        <v>10569.93598425169</v>
       </c>
       <c r="I10">
-        <v>199.0276841437618</v>
+        <v>198.651097844753</v>
       </c>
       <c r="J10">
-        <v>49.79252926758558</v>
+        <v>49.79208389066218</v>
       </c>
       <c r="K10">
-        <v>86.95085324866677</v>
+        <v>86.84602744570785</v>
       </c>
       <c r="L10">
-        <v>0.1908032720292201</v>
+        <v>0.1551236814572609</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -814,34 +814,34 @@
         <v>46296</v>
       </c>
       <c r="C11">
-        <v>58.03332213254248</v>
+        <v>74.86297397868663</v>
       </c>
       <c r="D11">
-        <v>232.1460501892969</v>
+        <v>232.4659537823925</v>
       </c>
       <c r="E11">
-        <v>36.54861744480475</v>
+        <v>36.30669207902036</v>
       </c>
       <c r="F11">
-        <v>0.6327282585570191</v>
+        <v>0.6240118272700201</v>
       </c>
       <c r="G11">
-        <v>41.90786990757745</v>
+        <v>50.80517086475414</v>
       </c>
       <c r="H11">
-        <v>10574.84520299115</v>
+        <v>10570.86615314667</v>
       </c>
       <c r="I11">
-        <v>198.6704203378997</v>
+        <v>198.7635752117183</v>
       </c>
       <c r="J11">
-        <v>49.79225991944117</v>
+        <v>49.79188189307028</v>
       </c>
       <c r="K11">
-        <v>86.88152129105538</v>
+        <v>86.94977406659692</v>
       </c>
       <c r="L11">
-        <v>0.183390516593083</v>
+        <v>0.1621412514316532</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -852,34 +852,34 @@
         <v>46327</v>
       </c>
       <c r="C12">
-        <v>58.11612339049373</v>
+        <v>57.3325619195251</v>
       </c>
       <c r="D12">
-        <v>232.467318790547</v>
+        <v>232.1417942282072</v>
       </c>
       <c r="E12">
-        <v>36.44959935924854</v>
+        <v>37.4372383340148</v>
       </c>
       <c r="F12">
-        <v>0.6240461887976237</v>
+        <v>0.6272337413958484</v>
       </c>
       <c r="G12">
-        <v>41.6781074314747</v>
+        <v>35</v>
       </c>
       <c r="H12">
-        <v>10570.90065096207</v>
+        <v>10574.56006287268</v>
       </c>
       <c r="I12">
-        <v>198.7612995016065</v>
+        <v>198.7638458247209</v>
       </c>
       <c r="J12">
-        <v>49.79267919812911</v>
+        <v>49.79196362283582</v>
       </c>
       <c r="K12">
-        <v>86.90921126040281</v>
+        <v>86.98050946956288</v>
       </c>
       <c r="L12">
-        <v>0.2049294079416336</v>
+        <v>0.1696465434949969</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -890,34 +890,34 @@
         <v>46357</v>
       </c>
       <c r="C13">
-        <v>58.03395374681705</v>
+        <v>59.34164605007472</v>
       </c>
       <c r="D13">
-        <v>232.4679440546195</v>
+        <v>232.1382680340778</v>
       </c>
       <c r="E13">
-        <v>36.73676408376586</v>
+        <v>36.32471046899472</v>
       </c>
       <c r="F13">
-        <v>0.6266821062761477</v>
+        <v>0.6312552476121882</v>
       </c>
       <c r="G13">
-        <v>42.69418634619002</v>
+        <v>37.95561668866811</v>
       </c>
       <c r="H13">
-        <v>10569.97076715846</v>
+        <v>10575.40177448836</v>
       </c>
       <c r="I13">
-        <v>199.0336000796761</v>
+        <v>198.7664819690946</v>
       </c>
       <c r="J13">
-        <v>49.79260847809475</v>
+        <v>49.79248463818619</v>
       </c>
       <c r="K13">
-        <v>86.97973672633796</v>
+        <v>86.89275573145488</v>
       </c>
       <c r="L13">
-        <v>0.1857139026679571</v>
+        <v>0.1577657090885378</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -928,34 +928,34 @@
         <v>46388</v>
       </c>
       <c r="C14">
-        <v>58.11342353506317</v>
+        <v>52.50405360417636</v>
       </c>
       <c r="D14">
-        <v>232.4684857720633</v>
+        <v>232.134261360169</v>
       </c>
       <c r="E14">
-        <v>36.63057292219486</v>
+        <v>37.28497400905117</v>
       </c>
       <c r="F14">
-        <v>0.6282439936543331</v>
+        <v>0.6295914936663943</v>
       </c>
       <c r="G14">
-        <v>41.67003393799702</v>
+        <v>58.34841520324428</v>
       </c>
       <c r="H14">
-        <v>10570.86910639741</v>
+        <v>10570.32145062267</v>
       </c>
       <c r="I14">
-        <v>198.7572257094421</v>
+        <v>198.762427078058</v>
       </c>
       <c r="J14">
-        <v>49.79237136286758</v>
+        <v>49.79271861344019</v>
       </c>
       <c r="K14">
-        <v>86.96042045520618</v>
+        <v>86.9526764743337</v>
       </c>
       <c r="L14">
-        <v>0.1986877353472729</v>
+        <v>0.1575324220375248</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -966,34 +966,34 @@
         <v>46419</v>
       </c>
       <c r="C15">
-        <v>58.03395374681705</v>
+        <v>55.84067301875714</v>
       </c>
       <c r="D15">
-        <v>232.4785903120053</v>
+        <v>232.4771253176626</v>
       </c>
       <c r="E15">
-        <v>36.49844626777791</v>
+        <v>37.21372297150082</v>
       </c>
       <c r="F15">
-        <v>0.6266914312219928</v>
+        <v>0.6240246841238719</v>
       </c>
       <c r="G15">
-        <v>42.12311401971797</v>
+        <v>63.2102784701158</v>
       </c>
       <c r="H15">
-        <v>10569.79343518435</v>
+        <v>10571.20947900621</v>
       </c>
       <c r="I15">
-        <v>198.7618055503594</v>
+        <v>198.9061140560813</v>
       </c>
       <c r="J15">
-        <v>49.79207598490156</v>
+        <v>49.79262124801635</v>
       </c>
       <c r="K15">
-        <v>87.00943656664994</v>
+        <v>86.92338900863881</v>
       </c>
       <c r="L15">
-        <v>0.190203764886226</v>
+        <v>0.1613440846841842</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -1004,34 +1004,34 @@
         <v>46447</v>
       </c>
       <c r="C16">
-        <v>58.03309755335288</v>
+        <v>57.67123372689964</v>
       </c>
       <c r="D16">
-        <v>232.1339411762648</v>
+        <v>232.4708454178957</v>
       </c>
       <c r="E16">
-        <v>37.50674373340907</v>
+        <v>37.49095520951517</v>
       </c>
       <c r="F16">
-        <v>0.6279246319294006</v>
+        <v>0.6231241872338341</v>
       </c>
       <c r="G16">
-        <v>41.71550257619626</v>
+        <v>35.75113279986432</v>
       </c>
       <c r="H16">
-        <v>10573.81522305098</v>
+        <v>10574.03983204292</v>
       </c>
       <c r="I16">
-        <v>198.9196607879384</v>
+        <v>198.760203256737</v>
       </c>
       <c r="J16">
-        <v>49.79230535805819</v>
+        <v>49.79237323017112</v>
       </c>
       <c r="K16">
-        <v>86.9276147849434</v>
+        <v>87.03747978121228</v>
       </c>
       <c r="L16">
-        <v>0.1974900561841187</v>
+        <v>0.1787097997131785</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -1042,34 +1042,34 @@
         <v>46478</v>
       </c>
       <c r="C17">
-        <v>58.03571795042549</v>
+        <v>62.04842622221469</v>
       </c>
       <c r="D17">
-        <v>232.1390114237976</v>
+        <v>232.1430649625258</v>
       </c>
       <c r="E17">
-        <v>36.54525849900476</v>
+        <v>36.31259715175638</v>
       </c>
       <c r="F17">
-        <v>0.6307517402698817</v>
+        <v>0.6275184165328469</v>
       </c>
       <c r="G17">
-        <v>43.14835138884885</v>
+        <v>44.51537465732475</v>
       </c>
       <c r="H17">
-        <v>10570.83500987111</v>
+        <v>10574.88384551303</v>
       </c>
       <c r="I17">
-        <v>198.8612078467727</v>
+        <v>198.8204509027399</v>
       </c>
       <c r="J17">
-        <v>49.79284176479196</v>
+        <v>49.79264119433672</v>
       </c>
       <c r="K17">
-        <v>86.78355556079603</v>
+        <v>87.01994007601563</v>
       </c>
       <c r="L17">
-        <v>0.1905019146140689</v>
+        <v>0.1568604758320835</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -1080,34 +1080,34 @@
         <v>46508</v>
       </c>
       <c r="C18">
-        <v>58.03427935560892</v>
+        <v>79.59338953815885</v>
       </c>
       <c r="D18">
-        <v>232.1329475749409</v>
+        <v>232.1365082772284</v>
       </c>
       <c r="E18">
-        <v>36.34100119759268</v>
+        <v>36.33173602183292</v>
       </c>
       <c r="F18">
-        <v>0.6269028110521925</v>
+        <v>0.627817372341211</v>
       </c>
       <c r="G18">
-        <v>41.70883637963371</v>
+        <v>39.7002501086267</v>
       </c>
       <c r="H18">
-        <v>10575.7257130516</v>
+        <v>10571.18879283526</v>
       </c>
       <c r="I18">
-        <v>198.660167686189</v>
+        <v>198.8083312782996</v>
       </c>
       <c r="J18">
-        <v>49.79244562264558</v>
+        <v>49.79195132510473</v>
       </c>
       <c r="K18">
-        <v>86.97106871318782</v>
+        <v>86.80846012118378</v>
       </c>
       <c r="L18">
-        <v>0.1887257260953796</v>
+        <v>0.1824685753212905</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -1118,34 +1118,34 @@
         <v>46539</v>
       </c>
       <c r="C19">
-        <v>58.03395374681705</v>
+        <v>58.10494295089483</v>
       </c>
       <c r="D19">
-        <v>232.1341235207319</v>
+        <v>232.4542391107396</v>
       </c>
       <c r="E19">
-        <v>36.248040267641</v>
+        <v>36.64572304253274</v>
       </c>
       <c r="F19">
-        <v>0.6255609963742642</v>
+        <v>0.6274318060294861</v>
       </c>
       <c r="G19">
-        <v>42.3318776006299</v>
+        <v>40.84201875770847</v>
       </c>
       <c r="H19">
-        <v>10569.95799239861</v>
+        <v>10570.90100979501</v>
       </c>
       <c r="I19">
-        <v>198.7188373221587</v>
+        <v>198.9051950848585</v>
       </c>
       <c r="J19">
-        <v>49.79297276542535</v>
+        <v>49.79264130668322</v>
       </c>
       <c r="K19">
-        <v>86.9161483944884</v>
+        <v>86.94539524107739</v>
       </c>
       <c r="L19">
-        <v>0.1934802123001007</v>
+        <v>0.171879634248835</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -1156,34 +1156,34 @@
         <v>46569</v>
       </c>
       <c r="C20">
-        <v>58.11985118913012</v>
+        <v>65.98595029839613</v>
       </c>
       <c r="D20">
-        <v>232.4530802619265</v>
+        <v>232.1406902229594</v>
       </c>
       <c r="E20">
-        <v>36.46148041486381</v>
+        <v>36.52727909103844</v>
       </c>
       <c r="F20">
-        <v>0.6327535025691281</v>
+        <v>0.6327371519396078</v>
       </c>
       <c r="G20">
-        <v>41.9967115903438</v>
+        <v>49.29141147547124</v>
       </c>
       <c r="H20">
-        <v>10571.17362718026</v>
+        <v>10570.3048362673</v>
       </c>
       <c r="I20">
-        <v>198.9488522282338</v>
+        <v>198.9236320188139</v>
       </c>
       <c r="J20">
-        <v>49.79248570749083</v>
+        <v>49.79277901020914</v>
       </c>
       <c r="K20">
-        <v>86.89194980541747</v>
+        <v>86.99395570986562</v>
       </c>
       <c r="L20">
-        <v>0.189718292673049</v>
+        <v>0.1776078926584725</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -1194,34 +1194,34 @@
         <v>46600</v>
       </c>
       <c r="C21">
-        <v>58.11328282159641</v>
+        <v>84.2831732786217</v>
       </c>
       <c r="D21">
-        <v>232.4530802619265</v>
+        <v>232.4565720652361</v>
       </c>
       <c r="E21">
-        <v>36.2007188546995</v>
+        <v>36.45335368365534</v>
       </c>
       <c r="F21">
-        <v>0.6259614545292138</v>
+        <v>0.6280616177863693</v>
       </c>
       <c r="G21">
-        <v>43.23929238682879</v>
+        <v>44.61015070958916</v>
       </c>
       <c r="H21">
-        <v>10574.31631458335</v>
+        <v>10574.79947862758</v>
       </c>
       <c r="I21">
-        <v>198.8840000568318</v>
+        <v>198.7740041531623</v>
       </c>
       <c r="J21">
-        <v>49.79282421566077</v>
+        <v>49.79308802215166</v>
       </c>
       <c r="K21">
-        <v>87.02337102205477</v>
+        <v>86.9678756604428</v>
       </c>
       <c r="L21">
-        <v>0.1941930074009073</v>
+        <v>0.1845134525258257</v>
       </c>
     </row>
     <row r="22" spans="1:12">
@@ -1232,34 +1232,34 @@
         <v>46631</v>
       </c>
       <c r="C22">
-        <v>58.1164141017934</v>
+        <v>46.83321430439985</v>
       </c>
       <c r="D22">
-        <v>232.4651652925421</v>
+        <v>232.4666973711687</v>
       </c>
       <c r="E22">
-        <v>36.5631550103592</v>
+        <v>36.23963590353537</v>
       </c>
       <c r="F22">
-        <v>0.6446406659074236</v>
+        <v>0.6426124162261481</v>
       </c>
       <c r="G22">
-        <v>41.63436749883052</v>
+        <v>51.79196211800782</v>
       </c>
       <c r="H22">
-        <v>10573.58913800262</v>
+        <v>10573.8140866053</v>
       </c>
       <c r="I22">
-        <v>198.9182173990962</v>
+        <v>198.9027323986821</v>
       </c>
       <c r="J22">
-        <v>49.79213905311308</v>
+        <v>49.79302652701128</v>
       </c>
       <c r="K22">
-        <v>86.87656897918818</v>
+        <v>86.81183501209898</v>
       </c>
       <c r="L22">
-        <v>0.1937032993774232</v>
+        <v>0.1759655813817785</v>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -1270,34 +1270,34 @@
         <v>46661</v>
       </c>
       <c r="C23">
-        <v>58.03510696097173</v>
+        <v>60.10225540227556</v>
       </c>
       <c r="D23">
-        <v>232.4512082177251</v>
+        <v>232.4697021201321</v>
       </c>
       <c r="E23">
-        <v>36.66274513563917</v>
+        <v>36.31259715175638</v>
       </c>
       <c r="F23">
-        <v>0.6347732443657693</v>
+        <v>0.6316763233136047</v>
       </c>
       <c r="G23">
-        <v>42.60681839116112</v>
+        <v>37.16510102508428</v>
       </c>
       <c r="H23">
-        <v>10573.6212245115</v>
+        <v>10573.9765312407</v>
       </c>
       <c r="I23">
-        <v>198.9242870147456</v>
+        <v>198.8523962594803</v>
       </c>
       <c r="J23">
-        <v>49.79232269268319</v>
+        <v>49.79208859966636</v>
       </c>
       <c r="K23">
-        <v>86.85603369879708</v>
+        <v>86.84148187593398</v>
       </c>
       <c r="L23">
-        <v>0.1909903042939717</v>
+        <v>0.1567639117239042</v>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -1308,34 +1308,34 @@
         <v>46692</v>
       </c>
       <c r="C24">
-        <v>58.12006515427251</v>
+        <v>58.76646892367128</v>
       </c>
       <c r="D24">
-        <v>232.1378640958966</v>
+        <v>232.1356764766872</v>
       </c>
       <c r="E24">
-        <v>36.50333240045298</v>
+        <v>36.41442432632038</v>
       </c>
       <c r="F24">
-        <v>0.6343696315013085</v>
+        <v>0.6267026400035168</v>
       </c>
       <c r="G24">
-        <v>43.07485436585291</v>
+        <v>36.1550497762799</v>
       </c>
       <c r="H24">
-        <v>10570.22522611249</v>
+        <v>10570.88273777708</v>
       </c>
       <c r="I24">
-        <v>199.0064420146134</v>
+        <v>198.90813891831</v>
       </c>
       <c r="J24">
-        <v>49.79246816290538</v>
+        <v>49.79296873747512</v>
       </c>
       <c r="K24">
-        <v>87.00765628823522</v>
+        <v>86.93478320739703</v>
       </c>
       <c r="L24">
-        <v>0.2015842715359286</v>
+        <v>0.1747451268286126</v>
       </c>
     </row>
     <row r="25" spans="1:12">
@@ -1346,34 +1346,34 @@
         <v>46722</v>
       </c>
       <c r="C25">
-        <v>58.11714013703779</v>
+        <v>65.57298706124259</v>
       </c>
       <c r="D25">
-        <v>232.4542392703406</v>
+        <v>232.4809856998034</v>
       </c>
       <c r="E25">
-        <v>36.48539941557534</v>
+        <v>36.46240376741557</v>
       </c>
       <c r="F25">
-        <v>0.6289693272406102</v>
+        <v>0.6260365811065993</v>
       </c>
       <c r="G25">
-        <v>41.71919070301217</v>
+        <v>49.2965780118875</v>
       </c>
       <c r="H25">
-        <v>10570.83308446542</v>
+        <v>10571.29042270445</v>
       </c>
       <c r="I25">
-        <v>198.6560277629817</v>
+        <v>198.7758829946662</v>
       </c>
       <c r="J25">
-        <v>49.79260319884644</v>
+        <v>49.7928422877154</v>
       </c>
       <c r="K25">
-        <v>87.00450539142768</v>
+        <v>87.01232598469761</v>
       </c>
       <c r="L25">
-        <v>0.1903193225856999</v>
+        <v>0.1642879366793548</v>
       </c>
     </row>
     <row r="26" spans="1:12">
@@ -1384,34 +1384,34 @@
         <v>46023</v>
       </c>
       <c r="C26">
-        <v>58.72874671229112</v>
+        <v>78.22888880543456</v>
       </c>
       <c r="D26">
-        <v>234.9153931730142</v>
+        <v>234.5882175612865</v>
       </c>
       <c r="E26">
-        <v>37.43883926390883</v>
+        <v>37.48829391072929</v>
       </c>
       <c r="F26">
-        <v>0.6312637364196606</v>
+        <v>0.6430658710211639</v>
       </c>
       <c r="G26">
-        <v>41.65383918840605</v>
+        <v>36.13620381522725</v>
       </c>
       <c r="H26">
-        <v>10575.10492579778</v>
+        <v>10574.44265223545</v>
       </c>
       <c r="I26">
-        <v>200.896477998705</v>
+        <v>201.1482075226983</v>
       </c>
       <c r="J26">
-        <v>49.79227545087875</v>
+        <v>49.79195835781121</v>
       </c>
       <c r="K26">
-        <v>87.4373212654947</v>
+        <v>87.31834647807513</v>
       </c>
       <c r="L26">
-        <v>0.1961384027107569</v>
+        <v>0.2452680977163396</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -1422,34 +1422,34 @@
         <v>46054</v>
       </c>
       <c r="C27">
-        <v>58.64695223805523</v>
+        <v>59.13246551446211</v>
       </c>
       <c r="D27">
-        <v>234.5915640885427</v>
+        <v>234.9319132389878</v>
       </c>
       <c r="E27">
-        <v>37.0262778056597</v>
+        <v>36.65863224525172</v>
       </c>
       <c r="F27">
-        <v>0.6314379187001555</v>
+        <v>0.6275599055576081</v>
       </c>
       <c r="G27">
-        <v>43.20125480987395</v>
+        <v>56.38121719969308</v>
       </c>
       <c r="H27">
-        <v>10574.65386370402</v>
+        <v>10574.19489635037</v>
       </c>
       <c r="I27">
-        <v>200.8971719877035</v>
+        <v>201.0539884382173</v>
       </c>
       <c r="J27">
-        <v>49.79327916074324</v>
+        <v>49.79302229527863</v>
       </c>
       <c r="K27">
-        <v>87.48472950455114</v>
+        <v>87.38295515074699</v>
       </c>
       <c r="L27">
-        <v>0.1813034588371743</v>
+        <v>0.2456428374002339</v>
       </c>
     </row>
     <row r="28" spans="1:12">
@@ -1460,34 +1460,34 @@
         <v>46082</v>
       </c>
       <c r="C28">
-        <v>58.64700864459076</v>
+        <v>56.5657936223981</v>
       </c>
       <c r="D28">
-        <v>234.5972972477312</v>
+        <v>234.9192306023454</v>
       </c>
       <c r="E28">
-        <v>37.13809877724496</v>
+        <v>36.88608533794548</v>
       </c>
       <c r="F28">
-        <v>0.6237526533252732</v>
+        <v>0.6276881912905959</v>
       </c>
       <c r="G28">
-        <v>42.37166624964006</v>
+        <v>46.47686112990034</v>
       </c>
       <c r="H28">
-        <v>10569.14620056335</v>
+        <v>10569.95094414414</v>
       </c>
       <c r="I28">
-        <v>200.7798739727429</v>
+        <v>200.9903696900552</v>
       </c>
       <c r="J28">
-        <v>49.79239127331684</v>
+        <v>49.7930233153056</v>
       </c>
       <c r="K28">
-        <v>87.41764999571899</v>
+        <v>87.48245088601935</v>
       </c>
       <c r="L28">
-        <v>0.2183763335127861</v>
+        <v>0.2070010442510791</v>
       </c>
     </row>
     <row r="29" spans="1:12">
@@ -1498,34 +1498,34 @@
         <v>46113</v>
       </c>
       <c r="C29">
-        <v>58.64696568776442</v>
+        <v>53.75000625615134</v>
       </c>
       <c r="D29">
-        <v>234.5945873935146</v>
+        <v>234.592681810285</v>
       </c>
       <c r="E29">
-        <v>37.27017466381513</v>
+        <v>36.66380402369808</v>
       </c>
       <c r="F29">
-        <v>0.6256223492901519</v>
+        <v>0.628093005808244</v>
       </c>
       <c r="G29">
-        <v>42.58456543894636</v>
+        <v>38.89503754345152</v>
       </c>
       <c r="H29">
-        <v>10570.14586358654</v>
+        <v>10574.23693964763</v>
       </c>
       <c r="I29">
-        <v>200.9436159546877</v>
+        <v>200.9111799981168</v>
       </c>
       <c r="J29">
-        <v>49.79222733451555</v>
+        <v>49.79154598357614</v>
       </c>
       <c r="K29">
-        <v>87.19593776724702</v>
+        <v>87.33407218204334</v>
       </c>
       <c r="L29">
-        <v>0.2067954173951712</v>
+        <v>0.2092509644240476</v>
       </c>
     </row>
     <row r="30" spans="1:12">
@@ -1536,34 +1536,34 @@
         <v>46143</v>
       </c>
       <c r="C30">
-        <v>58.72629317556929</v>
+        <v>60.62816001705295</v>
       </c>
       <c r="D30">
-        <v>234.9193206988262</v>
+        <v>234.9321878782433</v>
       </c>
       <c r="E30">
-        <v>36.66930908088512</v>
+        <v>36.82963438132322</v>
       </c>
       <c r="F30">
-        <v>0.6274582918478053</v>
+        <v>0.6350610460701455</v>
       </c>
       <c r="G30">
-        <v>41.61941310492224</v>
+        <v>35</v>
       </c>
       <c r="H30">
-        <v>10573.14342582038</v>
+        <v>10574.59543551355</v>
       </c>
       <c r="I30">
-        <v>201.0635846814714</v>
+        <v>201.1098872315088</v>
       </c>
       <c r="J30">
-        <v>49.79226345045905</v>
+        <v>49.79241536740415</v>
       </c>
       <c r="K30">
-        <v>87.49462793383219</v>
+        <v>87.3287431565292</v>
       </c>
       <c r="L30">
-        <v>0.2200516858371697</v>
+        <v>0.1910884069898511</v>
       </c>
     </row>
     <row r="31" spans="1:12">
@@ -1574,34 +1574,34 @@
         <v>46174</v>
       </c>
       <c r="C31">
-        <v>58.64687783814777</v>
+        <v>65.03974014137052</v>
       </c>
       <c r="D31">
-        <v>234.5895784713875</v>
+        <v>234.580588181669</v>
       </c>
       <c r="E31">
-        <v>36.76457378351024</v>
+        <v>37.72926126067836</v>
       </c>
       <c r="F31">
-        <v>0.6345833028033252</v>
+        <v>0.6265647586361389</v>
       </c>
       <c r="G31">
-        <v>41.60976267139159</v>
+        <v>41.89577836483249</v>
       </c>
       <c r="H31">
-        <v>10574.49375921011</v>
+        <v>10575.32040470852</v>
       </c>
       <c r="I31">
-        <v>201.0888534858115</v>
+        <v>201.067093743467</v>
       </c>
       <c r="J31">
-        <v>49.79246725494356</v>
+        <v>49.79206063151525</v>
       </c>
       <c r="K31">
-        <v>87.42341808088726</v>
+        <v>87.2242754852485</v>
       </c>
       <c r="L31">
-        <v>0.1862774526263378</v>
+        <v>0.189942864318598</v>
       </c>
     </row>
     <row r="32" spans="1:12">
@@ -1612,34 +1612,34 @@
         <v>46204</v>
       </c>
       <c r="C32">
-        <v>58.73034717436567</v>
+        <v>55.35453461139616</v>
       </c>
       <c r="D32">
-        <v>234.9195021880199</v>
+        <v>234.5871597232469</v>
       </c>
       <c r="E32">
-        <v>37.89047620607558</v>
+        <v>37.84212956219415</v>
       </c>
       <c r="F32">
-        <v>0.6423602728404078</v>
+        <v>0.6248698696887405</v>
       </c>
       <c r="G32">
-        <v>41.91889528089124</v>
+        <v>54.44287858306039</v>
       </c>
       <c r="H32">
-        <v>10570.02580229721</v>
+        <v>10570.5101778998</v>
       </c>
       <c r="I32">
-        <v>200.931796009754</v>
+        <v>200.994166650209</v>
       </c>
       <c r="J32">
-        <v>49.79258941346781</v>
+        <v>49.79287460201898</v>
       </c>
       <c r="K32">
-        <v>87.4693687689802</v>
+        <v>87.42593663050805</v>
       </c>
       <c r="L32">
-        <v>0.2207172385116133</v>
+        <v>0.2205403207637926</v>
       </c>
     </row>
     <row r="33" spans="1:12">
@@ -1650,34 +1650,34 @@
         <v>46235</v>
       </c>
       <c r="C33">
-        <v>58.72971281486267</v>
+        <v>53.84807239076564</v>
       </c>
       <c r="D33">
-        <v>234.591168154171</v>
+        <v>234.5846280459897</v>
       </c>
       <c r="E33">
-        <v>36.96950773455673</v>
+        <v>36.97163614467719</v>
       </c>
       <c r="F33">
-        <v>0.6244622746769143</v>
+        <v>0.6249093895315039</v>
       </c>
       <c r="G33">
-        <v>43.1149277801069</v>
+        <v>58.91638449973042</v>
       </c>
       <c r="H33">
-        <v>10569.39443385744</v>
+        <v>10575.1999964891</v>
       </c>
       <c r="I33">
-        <v>201.1165798297785</v>
+        <v>200.7898853651306</v>
       </c>
       <c r="J33">
-        <v>49.79253983225752</v>
+        <v>49.79248490464077</v>
       </c>
       <c r="K33">
-        <v>87.49843410838854</v>
+        <v>87.30050820119212</v>
       </c>
       <c r="L33">
-        <v>0.214482631101949</v>
+        <v>0.2122599541793017</v>
       </c>
     </row>
     <row r="34" spans="1:12">
@@ -1688,34 +1688,34 @@
         <v>46266</v>
       </c>
       <c r="C34">
-        <v>58.72653570857705</v>
+        <v>78.95628851239331</v>
       </c>
       <c r="D34">
-        <v>234.9193206988262</v>
+        <v>234.5868897758578</v>
       </c>
       <c r="E34">
-        <v>36.77762613017127</v>
+        <v>37.21469498554619</v>
       </c>
       <c r="F34">
-        <v>0.6242453618951807</v>
+        <v>0.6258103352215929</v>
       </c>
       <c r="G34">
-        <v>42.15799731374506</v>
+        <v>53.91960905044375</v>
       </c>
       <c r="H34">
-        <v>10574.49011217136</v>
+        <v>10575.32040470852</v>
       </c>
       <c r="I34">
-        <v>201.1111199994134</v>
+        <v>201.0217504115023</v>
       </c>
       <c r="J34">
-        <v>49.79329382748796</v>
+        <v>49.79240544152003</v>
       </c>
       <c r="K34">
-        <v>87.43264979206583</v>
+        <v>87.28956163119915</v>
       </c>
       <c r="L34">
-        <v>0.1961384027107569</v>
+        <v>0.247657392387849</v>
       </c>
     </row>
     <row r="35" spans="1:12">
@@ -1726,34 +1726,34 @@
         <v>46296</v>
       </c>
       <c r="C35">
-        <v>58.64615246056417</v>
+        <v>61.5159018004289</v>
       </c>
       <c r="D35">
-        <v>234.9072893439312</v>
+        <v>234.592681810285</v>
       </c>
       <c r="E35">
-        <v>36.71488490609664</v>
+        <v>36.70575912251815</v>
       </c>
       <c r="F35">
-        <v>0.6320221120744065</v>
+        <v>0.626819618421216</v>
       </c>
       <c r="G35">
-        <v>41.86930941371875</v>
+        <v>53.6579761652584</v>
       </c>
       <c r="H35">
-        <v>10569.5770516864</v>
+        <v>10574.39007159036</v>
       </c>
       <c r="I35">
-        <v>200.9117546189998</v>
+        <v>200.9184664969263</v>
       </c>
       <c r="J35">
-        <v>49.79276110127992</v>
+        <v>49.79275117127339</v>
       </c>
       <c r="K35">
-        <v>87.35983432206656</v>
+        <v>87.37249139312189</v>
       </c>
       <c r="L35">
-        <v>0.1914043654359489</v>
+        <v>0.2460216319573676</v>
       </c>
     </row>
     <row r="36" spans="1:12">
@@ -1764,34 +1764,34 @@
         <v>46327</v>
       </c>
       <c r="C36">
-        <v>58.72958054826571</v>
+        <v>57.83501026344599</v>
       </c>
       <c r="D36">
-        <v>234.9311055947933</v>
+        <v>234.9156813322722</v>
       </c>
       <c r="E36">
-        <v>36.83256664142496</v>
+        <v>37.49719145176856</v>
       </c>
       <c r="F36">
-        <v>0.6288385248819104</v>
+        <v>0.6322647420270098</v>
       </c>
       <c r="G36">
-        <v>41.87899291349752</v>
+        <v>38.75452613542967</v>
       </c>
       <c r="H36">
-        <v>10575.46353441383</v>
+        <v>10575.70025954445</v>
       </c>
       <c r="I36">
-        <v>201.001499734509</v>
+        <v>201.0286624009604</v>
       </c>
       <c r="J36">
-        <v>49.79325570844328</v>
+        <v>49.79239380217934</v>
       </c>
       <c r="K36">
-        <v>87.48904836845382</v>
+        <v>87.18824481318606</v>
       </c>
       <c r="L36">
-        <v>0.2014398527546301</v>
+        <v>0.2195823221139543</v>
       </c>
     </row>
     <row r="37" spans="1:12">
@@ -1802,34 +1802,34 @@
         <v>46357</v>
       </c>
       <c r="C37">
-        <v>58.64796102945098</v>
+        <v>60.84773720002896</v>
       </c>
       <c r="D37">
-        <v>234.8886502307469</v>
+        <v>234.5868897758578</v>
       </c>
       <c r="E37">
-        <v>36.7044177614645</v>
+        <v>36.98352180826824</v>
       </c>
       <c r="F37">
-        <v>0.6260362945774599</v>
+        <v>0.625838971273461</v>
       </c>
       <c r="G37">
-        <v>42.59123727823345</v>
+        <v>41.19113553804491</v>
       </c>
       <c r="H37">
-        <v>10573.0455992265</v>
+        <v>10574.36212128547</v>
       </c>
       <c r="I37">
-        <v>200.8915515873299</v>
+        <v>201.1320971419786</v>
       </c>
       <c r="J37">
-        <v>49.79278515231464</v>
+        <v>49.79285994785267</v>
       </c>
       <c r="K37">
-        <v>87.20037344536586</v>
+        <v>87.38208633012897</v>
       </c>
       <c r="L37">
-        <v>0.2190763335496272</v>
+        <v>0.1946075725560199</v>
       </c>
     </row>
     <row r="38" spans="1:12">
@@ -1840,34 +1840,34 @@
         <v>46388</v>
       </c>
       <c r="C38">
-        <v>58.72992190887436</v>
+        <v>46.31099633365717</v>
       </c>
       <c r="D38">
-        <v>234.7669562342057</v>
+        <v>234.5849613498855</v>
       </c>
       <c r="E38">
-        <v>36.8546333211517</v>
+        <v>37.05910863676856</v>
       </c>
       <c r="F38">
-        <v>0.6259685019070207</v>
+        <v>0.6264519091125674</v>
       </c>
       <c r="G38">
-        <v>41.80122290890426</v>
+        <v>66.34116726100194</v>
       </c>
       <c r="H38">
-        <v>10569.29056329186</v>
+        <v>10574.42809782194</v>
       </c>
       <c r="I38">
-        <v>200.9028807660497</v>
+        <v>201.0595137143139</v>
       </c>
       <c r="J38">
-        <v>49.79259813106679</v>
+        <v>49.79215071459365</v>
       </c>
       <c r="K38">
-        <v>87.49354869196118</v>
+        <v>87.43576701150313</v>
       </c>
       <c r="L38">
-        <v>0.2035465308840684</v>
+        <v>0.1924884882387086</v>
       </c>
     </row>
     <row r="39" spans="1:12">
@@ -1878,34 +1878,34 @@
         <v>46419</v>
       </c>
       <c r="C39">
-        <v>58.73219980608017</v>
+        <v>65.1049221401006</v>
       </c>
       <c r="D39">
-        <v>234.9060950792406</v>
+        <v>234.9223285214258</v>
       </c>
       <c r="E39">
-        <v>36.82270194054684</v>
+        <v>36.74426085163817</v>
       </c>
       <c r="F39">
-        <v>0.6285230195302863</v>
+        <v>0.6242277975290497</v>
       </c>
       <c r="G39">
-        <v>41.82464304649142</v>
+        <v>35</v>
       </c>
       <c r="H39">
-        <v>10574.92700505827</v>
+        <v>10571.15619012403</v>
       </c>
       <c r="I39">
-        <v>201.0978482469702</v>
+        <v>201.0620374143748</v>
       </c>
       <c r="J39">
-        <v>49.79294858017524</v>
+        <v>49.79280567018966</v>
       </c>
       <c r="K39">
-        <v>87.30982509152442</v>
+        <v>87.43291931213733</v>
       </c>
       <c r="L39">
-        <v>0.2120104373711515</v>
+        <v>0.2189528503820617</v>
       </c>
     </row>
     <row r="40" spans="1:12">
@@ -1916,34 +1916,34 @@
         <v>46447</v>
       </c>
       <c r="C40">
-        <v>58.73318186074254</v>
+        <v>62.10045688235381</v>
       </c>
       <c r="D40">
-        <v>234.9164443251064</v>
+        <v>234.9218238812649</v>
       </c>
       <c r="E40">
-        <v>36.74753755320991</v>
+        <v>37.91821174059719</v>
       </c>
       <c r="F40">
-        <v>0.6492763842041803</v>
+        <v>0.6271501059284558</v>
       </c>
       <c r="G40">
-        <v>42.45934483040212</v>
+        <v>35</v>
       </c>
       <c r="H40">
-        <v>10573.14563454924</v>
+        <v>10570.14464027459</v>
       </c>
       <c r="I40">
-        <v>200.8872617162509</v>
+        <v>200.9992347897689</v>
       </c>
       <c r="J40">
-        <v>49.79344787256795</v>
+        <v>49.79184996161249</v>
       </c>
       <c r="K40">
-        <v>87.42580641752858</v>
+        <v>87.36362626182695</v>
       </c>
       <c r="L40">
-        <v>0.1971962993531581</v>
+        <v>0.209860551973115</v>
       </c>
     </row>
     <row r="41" spans="1:12">
@@ -1954,34 +1954,34 @@
         <v>46478</v>
       </c>
       <c r="C41">
-        <v>58.64732119431034</v>
+        <v>76.2792148871869</v>
       </c>
       <c r="D41">
-        <v>234.9072893439312</v>
+        <v>234.5935726745974</v>
       </c>
       <c r="E41">
-        <v>37.21314336658764</v>
+        <v>36.78938824887655</v>
       </c>
       <c r="F41">
-        <v>0.6293100692325327</v>
+        <v>0.6267534717904528</v>
       </c>
       <c r="G41">
-        <v>42.38913360322601</v>
+        <v>63.56382864043049</v>
       </c>
       <c r="H41">
-        <v>10573.01713501526</v>
+        <v>10571.17507024421</v>
       </c>
       <c r="I41">
-        <v>200.96239301264</v>
+        <v>200.7913136343865</v>
       </c>
       <c r="J41">
-        <v>49.79259165302766</v>
+        <v>49.79225730697006</v>
       </c>
       <c r="K41">
-        <v>87.24895446602979</v>
+        <v>87.36797778076595</v>
       </c>
       <c r="L41">
-        <v>0.1827668252189182</v>
+        <v>0.2094056590845625</v>
       </c>
     </row>
     <row r="42" spans="1:12">
@@ -1992,34 +1992,34 @@
         <v>46508</v>
       </c>
       <c r="C42">
-        <v>58.72692322962403</v>
+        <v>63.92097234311526</v>
       </c>
       <c r="D42">
-        <v>234.5851362680061</v>
+        <v>234.9219631951441</v>
       </c>
       <c r="E42">
-        <v>37.77236183071258</v>
+        <v>36.87023438640199</v>
       </c>
       <c r="F42">
-        <v>0.6246929988330319</v>
+        <v>0.6268308232189056</v>
       </c>
       <c r="G42">
-        <v>41.71244722523189</v>
+        <v>52.87677133303077</v>
       </c>
       <c r="H42">
-        <v>10575.33645065357</v>
+        <v>10574.86543627049</v>
       </c>
       <c r="I42">
-        <v>200.9875364356983</v>
+        <v>200.9329997120207</v>
       </c>
       <c r="J42">
-        <v>49.79286429815082</v>
+        <v>49.79240343234689</v>
       </c>
       <c r="K42">
-        <v>87.3251585997734</v>
+        <v>87.44187449017231</v>
       </c>
       <c r="L42">
-        <v>0.1915770921330487</v>
+        <v>0.2076563576605265</v>
       </c>
     </row>
     <row r="43" spans="1:12">
@@ -2030,34 +2030,34 @@
         <v>46539</v>
       </c>
       <c r="C43">
-        <v>58.73042239906079</v>
+        <v>44.25228206818315</v>
       </c>
       <c r="D43">
-        <v>234.9182342035807</v>
+        <v>234.5834716616997</v>
       </c>
       <c r="E43">
-        <v>36.77047716528153</v>
+        <v>36.78204673239873</v>
       </c>
       <c r="F43">
-        <v>0.6241566269698848</v>
+        <v>0.6251708672623645</v>
       </c>
       <c r="G43">
-        <v>41.89057819605816</v>
+        <v>42.05800206379978</v>
       </c>
       <c r="H43">
-        <v>10573.14060511415</v>
+        <v>10576.25159810396</v>
       </c>
       <c r="I43">
-        <v>201.0065748391279</v>
+        <v>200.8259024014877</v>
       </c>
       <c r="J43">
-        <v>49.79166859218383</v>
+        <v>49.79143500990446</v>
       </c>
       <c r="K43">
-        <v>87.51785142491811</v>
+        <v>87.45880508940017</v>
       </c>
       <c r="L43">
-        <v>0.1886809333452674</v>
+        <v>0.211373496854876</v>
       </c>
     </row>
     <row r="44" spans="1:12">
@@ -2068,34 +2068,34 @@
         <v>46569</v>
       </c>
       <c r="C44">
-        <v>58.64715663359507</v>
+        <v>57.33927346595685</v>
       </c>
       <c r="D44">
-        <v>234.906544467887</v>
+        <v>234.5868897758578</v>
       </c>
       <c r="E44">
-        <v>37.52761287636463</v>
+        <v>37.21766029196537</v>
       </c>
       <c r="F44">
-        <v>0.627419177165991</v>
+        <v>0.6247573812708347</v>
       </c>
       <c r="G44">
-        <v>43.35040199581663</v>
+        <v>60.19831627713235</v>
       </c>
       <c r="H44">
-        <v>10573.25906946188</v>
+        <v>10571.16807718535</v>
       </c>
       <c r="I44">
-        <v>201.0069198965132</v>
+        <v>200.7914521459456</v>
       </c>
       <c r="J44">
-        <v>49.79236040000348</v>
+        <v>49.79192595029681</v>
       </c>
       <c r="K44">
-        <v>87.34621349506676</v>
+        <v>87.39037474444959</v>
       </c>
       <c r="L44">
-        <v>0.1799139160735753</v>
+        <v>0.1919690596400888</v>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -2106,34 +2106,34 @@
         <v>46600</v>
       </c>
       <c r="C45">
-        <v>58.64672458158702</v>
+        <v>59.73394196457834</v>
       </c>
       <c r="D45">
-        <v>234.9054782404973</v>
+        <v>234.5866199980599</v>
       </c>
       <c r="E45">
-        <v>37.4878731167981</v>
+        <v>36.94624404494752</v>
       </c>
       <c r="F45">
-        <v>0.6360189850042989</v>
+        <v>0.6469510592761505</v>
       </c>
       <c r="G45">
-        <v>41.65324327740931</v>
+        <v>35</v>
       </c>
       <c r="H45">
-        <v>10570.09597953125</v>
+        <v>10570.72647108511</v>
       </c>
       <c r="I45">
-        <v>200.7754437784296</v>
+        <v>200.7778844904458</v>
       </c>
       <c r="J45">
-        <v>49.79293695495755</v>
+        <v>49.79274449550525</v>
       </c>
       <c r="K45">
-        <v>87.41909061822284</v>
+        <v>87.50065642435574</v>
       </c>
       <c r="L45">
-        <v>0.2233498235507761</v>
+        <v>0.2341835770230538</v>
       </c>
     </row>
     <row r="46" spans="1:12">
@@ -2144,34 +2144,34 @@
         <v>46631</v>
       </c>
       <c r="C46">
-        <v>58.72677757712942</v>
+        <v>53.29227110962166</v>
       </c>
       <c r="D46">
-        <v>234.5928030398842</v>
+        <v>234.9077347989345</v>
       </c>
       <c r="E46">
-        <v>37.69024745343437</v>
+        <v>38.12799698903888</v>
       </c>
       <c r="F46">
-        <v>0.624522986539981</v>
+        <v>0.6279855283780094</v>
       </c>
       <c r="G46">
-        <v>42.00487584183178</v>
+        <v>35</v>
       </c>
       <c r="H46">
-        <v>10569.7706699247</v>
+        <v>10574.77545133333</v>
       </c>
       <c r="I46">
-        <v>201.0295565333922</v>
+        <v>201.0001885882679</v>
       </c>
       <c r="J46">
-        <v>49.79198850670367</v>
+        <v>49.79267316583973</v>
       </c>
       <c r="K46">
-        <v>87.39001014822512</v>
+        <v>87.40559430091267</v>
       </c>
       <c r="L46">
-        <v>0.1964287088237587</v>
+        <v>0.2128031645195091</v>
       </c>
     </row>
     <row r="47" spans="1:12">
@@ -2182,34 +2182,34 @@
         <v>46661</v>
       </c>
       <c r="C47">
-        <v>58.73328525317118</v>
+        <v>76.88693720902691</v>
       </c>
       <c r="D47">
-        <v>234.5911881874789</v>
+        <v>234.9218238812649</v>
       </c>
       <c r="E47">
-        <v>37.75776207632661</v>
+        <v>36.61516720845789</v>
       </c>
       <c r="F47">
-        <v>0.6266533018613113</v>
+        <v>0.6279688772354034</v>
       </c>
       <c r="G47">
-        <v>41.67053048260343</v>
+        <v>53.0273913365269</v>
       </c>
       <c r="H47">
-        <v>10573.23829010507</v>
+        <v>10570.46487593437</v>
       </c>
       <c r="I47">
-        <v>200.906315122388</v>
+        <v>201.1201007406279</v>
       </c>
       <c r="J47">
-        <v>49.79293303933099</v>
+        <v>49.79135954427056</v>
       </c>
       <c r="K47">
-        <v>87.39250868729863</v>
+        <v>87.23854567882559</v>
       </c>
       <c r="L47">
-        <v>0.1799073397844037</v>
+        <v>0.2341846943019588</v>
       </c>
     </row>
     <row r="48" spans="1:12">
@@ -2220,34 +2220,34 @@
         <v>46692</v>
       </c>
       <c r="C48">
-        <v>58.64641810526948</v>
+        <v>57.69448909891042</v>
       </c>
       <c r="D48">
-        <v>234.5949627599814</v>
+        <v>234.9318465779948</v>
       </c>
       <c r="E48">
-        <v>36.84664481626714</v>
+        <v>37.09692053806557</v>
       </c>
       <c r="F48">
-        <v>0.6251046070230637</v>
+        <v>0.6429626951342748</v>
       </c>
       <c r="G48">
-        <v>43.2014698715757</v>
+        <v>50.39214237806548</v>
       </c>
       <c r="H48">
-        <v>10569.50318854462</v>
+        <v>10570.90439582538</v>
       </c>
       <c r="I48">
-        <v>201.007349730879</v>
+        <v>200.9318412543039</v>
       </c>
       <c r="J48">
-        <v>49.79296027539214</v>
+        <v>49.7919419338818</v>
       </c>
       <c r="K48">
-        <v>87.27395954666127</v>
+        <v>87.42593663050805</v>
       </c>
       <c r="L48">
-        <v>0.2130720164791403</v>
+        <v>0.2096447036054359</v>
       </c>
     </row>
     <row r="49" spans="1:12">
@@ -2258,34 +2258,34 @@
         <v>46722</v>
       </c>
       <c r="C49">
-        <v>58.73325622317398</v>
+        <v>55.78002587386893</v>
       </c>
       <c r="D49">
-        <v>234.9315694882112</v>
+        <v>234.9052617462014</v>
       </c>
       <c r="E49">
-        <v>37.41723364210234</v>
+        <v>37.87211014927965</v>
       </c>
       <c r="F49">
-        <v>0.6301774841608382</v>
+        <v>0.624319661756608</v>
       </c>
       <c r="G49">
-        <v>41.94242393867813</v>
+        <v>40.61573749691113</v>
       </c>
       <c r="H49">
-        <v>10569.50318854462</v>
+        <v>10570.98840124256</v>
       </c>
       <c r="I49">
-        <v>200.890530828446</v>
+        <v>201.0459295734242</v>
       </c>
       <c r="J49">
-        <v>49.79255301836432</v>
+        <v>49.79319130057611</v>
       </c>
       <c r="K49">
-        <v>87.348356557055</v>
+        <v>87.30980053729729</v>
       </c>
       <c r="L49">
-        <v>0.1839034809843912</v>
+        <v>0.1743897367086141</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -2296,34 +2296,34 @@
         <v>46023</v>
       </c>
       <c r="C50">
-        <v>59.94509744742375</v>
+        <v>58.7982080838774</v>
       </c>
       <c r="D50">
-        <v>239.7928512258672</v>
+        <v>239.4572256458415</v>
       </c>
       <c r="E50">
-        <v>37.70943902510526</v>
+        <v>37.44244605806163</v>
       </c>
       <c r="F50">
-        <v>0.6243744006451795</v>
+        <v>0.6252002167722375</v>
       </c>
       <c r="G50">
-        <v>42.03945385771092</v>
+        <v>55.20622062062456</v>
       </c>
       <c r="H50">
-        <v>10574.84854099255</v>
+        <v>10576.12730503696</v>
       </c>
       <c r="I50">
-        <v>205.1818250739205</v>
+        <v>205.2366719142538</v>
       </c>
       <c r="J50">
-        <v>49.79232325667488</v>
+        <v>49.79255686840897</v>
       </c>
       <c r="K50">
-        <v>88.27321103056234</v>
+        <v>88.39547605135911</v>
       </c>
       <c r="L50">
-        <v>0.2199453164743143</v>
+        <v>0.2036814258674093</v>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -2334,34 +2334,34 @@
         <v>46054</v>
       </c>
       <c r="C51">
-        <v>59.94542832387302</v>
+        <v>56.27814312482789</v>
       </c>
       <c r="D51">
-        <v>239.4579784662421</v>
+        <v>239.4550823770878</v>
       </c>
       <c r="E51">
-        <v>37.84291784216649</v>
+        <v>38.47988496270941</v>
       </c>
       <c r="F51">
-        <v>0.6441214726684734</v>
+        <v>0.6251535718648294</v>
       </c>
       <c r="G51">
-        <v>41.96301250684883</v>
+        <v>41.19604157122829</v>
       </c>
       <c r="H51">
-        <v>10574.17052082084</v>
+        <v>10569.72156615773</v>
       </c>
       <c r="I51">
-        <v>205.0555579844585</v>
+        <v>205.0823281293985</v>
       </c>
       <c r="J51">
-        <v>49.79218912578737</v>
+        <v>49.79264247561623</v>
       </c>
       <c r="K51">
-        <v>88.38204227688283</v>
+        <v>88.14069678410415</v>
       </c>
       <c r="L51">
-        <v>0.2067519410122159</v>
+        <v>0.2037741193344408</v>
       </c>
     </row>
     <row r="52" spans="1:12">
@@ -2372,34 +2372,34 @@
         <v>46082</v>
       </c>
       <c r="C52">
-        <v>59.86388997763411</v>
+        <v>57.84868541148031</v>
       </c>
       <c r="D52">
-        <v>239.7778506036868</v>
+        <v>239.8075317588012</v>
       </c>
       <c r="E52">
-        <v>37.53124527870752</v>
+        <v>37.47813219819105</v>
       </c>
       <c r="F52">
-        <v>0.6305964361982329</v>
+        <v>0.6429039343734726</v>
       </c>
       <c r="G52">
-        <v>41.65515719554102</v>
+        <v>48.31301250972208</v>
       </c>
       <c r="H52">
-        <v>10573.19139744471</v>
+        <v>10570.52692994756</v>
       </c>
       <c r="I52">
-        <v>205.2703242955257</v>
+        <v>204.9415787183751</v>
       </c>
       <c r="J52">
-        <v>49.79245384355541</v>
+        <v>49.79265588222938</v>
       </c>
       <c r="K52">
-        <v>88.34577750635542</v>
+        <v>88.30493562844947</v>
       </c>
       <c r="L52">
-        <v>0.2283659084217927</v>
+        <v>0.2347955427893793</v>
       </c>
     </row>
     <row r="53" spans="1:12">
@@ -2410,34 +2410,34 @@
         <v>46113</v>
       </c>
       <c r="C53">
-        <v>59.86393095760406</v>
+        <v>53.22467309432027</v>
       </c>
       <c r="D53">
-        <v>239.7948178935006</v>
+        <v>239.7821228208283</v>
       </c>
       <c r="E53">
-        <v>37.44792096161357</v>
+        <v>37.5359150492064</v>
       </c>
       <c r="F53">
-        <v>0.6241564915328423</v>
+        <v>0.6270585966303197</v>
       </c>
       <c r="G53">
-        <v>41.93159790391319</v>
+        <v>59.86947454889263</v>
       </c>
       <c r="H53">
-        <v>10572.88612160042</v>
+        <v>10569.88991164868</v>
       </c>
       <c r="I53">
-        <v>205.1757780078244</v>
+        <v>205.1045686036013</v>
       </c>
       <c r="J53">
-        <v>49.79245567668748</v>
+        <v>49.792847873898</v>
       </c>
       <c r="K53">
-        <v>88.28909607413692</v>
+        <v>88.26000584003995</v>
       </c>
       <c r="L53">
-        <v>0.2202054485008916</v>
+        <v>0.2259128838616332</v>
       </c>
     </row>
     <row r="54" spans="1:12">
@@ -2448,34 +2448,34 @@
         <v>46143</v>
       </c>
       <c r="C54">
-        <v>59.9483539943143</v>
+        <v>53.57073843787349</v>
       </c>
       <c r="D54">
-        <v>239.8025590869516</v>
+        <v>239.4517293301137</v>
       </c>
       <c r="E54">
-        <v>38.12670119694982</v>
+        <v>37.40834189346466</v>
       </c>
       <c r="F54">
-        <v>0.623935858122707</v>
+        <v>0.6447758312724252</v>
       </c>
       <c r="G54">
-        <v>41.84085849184089</v>
+        <v>47.70248790155674</v>
       </c>
       <c r="H54">
-        <v>10570.64500732657</v>
+        <v>10571.86863408603</v>
       </c>
       <c r="I54">
-        <v>205.1987587514595</v>
+        <v>205.0969615853106</v>
       </c>
       <c r="J54">
-        <v>49.79253561992997</v>
+        <v>49.79167418490476</v>
       </c>
       <c r="K54">
-        <v>88.34575516383217</v>
+        <v>88.40463908238377</v>
       </c>
       <c r="L54">
-        <v>0.2218844785763742</v>
+        <v>0.2124396313093488</v>
       </c>
     </row>
     <row r="55" spans="1:12">
@@ -2486,34 +2486,34 @@
         <v>46174</v>
       </c>
       <c r="C55">
-        <v>59.86262930432519</v>
+        <v>64.16952855122651</v>
       </c>
       <c r="D55">
-        <v>239.7947851446239</v>
+        <v>239.4536690126795</v>
       </c>
       <c r="E55">
-        <v>37.52287083888366</v>
+        <v>38.3581502632396</v>
       </c>
       <c r="F55">
-        <v>0.6276537868796065</v>
+        <v>0.6358019413493711</v>
       </c>
       <c r="G55">
-        <v>42.7080802495874</v>
+        <v>46.2429221812957</v>
       </c>
       <c r="H55">
-        <v>10570.83254297152</v>
+        <v>10574.84018128014</v>
       </c>
       <c r="I55">
-        <v>205.1869091317443</v>
+        <v>205.1647923065301</v>
       </c>
       <c r="J55">
-        <v>49.793167305037</v>
+        <v>49.79194068737782</v>
       </c>
       <c r="K55">
-        <v>88.32932243845084</v>
+        <v>88.25653042751009</v>
       </c>
       <c r="L55">
-        <v>0.2071751826363247</v>
+        <v>0.2288640022241817</v>
       </c>
     </row>
     <row r="56" spans="1:12">
@@ -2524,34 +2524,34 @@
         <v>46204</v>
       </c>
       <c r="C56">
-        <v>59.94872000799104</v>
+        <v>66.39116337651375</v>
       </c>
       <c r="D56">
-        <v>239.7946219443304</v>
+        <v>239.7779384323789</v>
       </c>
       <c r="E56">
-        <v>37.88187016023065</v>
+        <v>37.38768551979406</v>
       </c>
       <c r="F56">
-        <v>0.6245499330669964</v>
+        <v>0.6254425475059485</v>
       </c>
       <c r="G56">
-        <v>42.45015746730273</v>
+        <v>55.52917235689421</v>
       </c>
       <c r="H56">
-        <v>10574.82224550185</v>
+        <v>10574.61651980317</v>
       </c>
       <c r="I56">
-        <v>204.930726161743</v>
+        <v>205.0844023845509</v>
       </c>
       <c r="J56">
-        <v>49.79226651163269</v>
+        <v>49.79280521378968</v>
       </c>
       <c r="K56">
-        <v>88.23348985500725</v>
+        <v>88.33877353457321</v>
       </c>
       <c r="L56">
-        <v>0.2265510480316036</v>
+        <v>0.2243873018204921</v>
       </c>
     </row>
     <row r="57" spans="1:12">
@@ -2562,34 +2562,34 @@
         <v>46235</v>
       </c>
       <c r="C57">
-        <v>59.94555652505674</v>
+        <v>61.65725802984672</v>
       </c>
       <c r="D57">
-        <v>239.4507657470699</v>
+        <v>239.7819017266507</v>
       </c>
       <c r="E57">
-        <v>37.4402491569595</v>
+        <v>37.85603541648712</v>
       </c>
       <c r="F57">
-        <v>0.6291821815044522</v>
+        <v>0.6323327587886305</v>
       </c>
       <c r="G57">
-        <v>42.78964049431111</v>
+        <v>48.36959051896095</v>
       </c>
       <c r="H57">
-        <v>10574.28641117162</v>
+        <v>10574.17736654278</v>
       </c>
       <c r="I57">
-        <v>204.9420025699181</v>
+        <v>205.2627336905961</v>
       </c>
       <c r="J57">
-        <v>49.79300778459324</v>
+        <v>49.79215753053039</v>
       </c>
       <c r="K57">
-        <v>88.1123716856923</v>
+        <v>88.34940499525689</v>
       </c>
       <c r="L57">
-        <v>0.2350250123805601</v>
+        <v>0.2257562837364423</v>
       </c>
     </row>
     <row r="58" spans="1:12">
@@ -2600,34 +2600,34 @@
         <v>46266</v>
       </c>
       <c r="C58">
-        <v>59.86254863503917</v>
+        <v>77.66205675054387</v>
       </c>
       <c r="D58">
-        <v>239.6629995791283</v>
+        <v>239.4511793956276</v>
       </c>
       <c r="E58">
-        <v>37.75424261405774</v>
+        <v>37.65268580776845</v>
       </c>
       <c r="F58">
-        <v>0.6371473612884938</v>
+        <v>0.6374701285098795</v>
       </c>
       <c r="G58">
-        <v>41.64335561361196</v>
+        <v>60.44612129420005</v>
       </c>
       <c r="H58">
-        <v>10570.92418027073</v>
+        <v>10570.36591931128</v>
       </c>
       <c r="I58">
-        <v>205.1717520476376</v>
+        <v>205.107953406127</v>
       </c>
       <c r="J58">
-        <v>49.79297824833746</v>
+        <v>49.79264092715604</v>
       </c>
       <c r="K58">
-        <v>88.32561966955758</v>
+        <v>88.42608135060779</v>
       </c>
       <c r="L58">
-        <v>0.2093004720717208</v>
+        <v>0.2023459506904151</v>
       </c>
     </row>
     <row r="59" spans="1:12">
@@ -2638,34 +2638,34 @@
         <v>46296</v>
       </c>
       <c r="C59">
-        <v>59.8644458883741</v>
+        <v>59.03223623184852</v>
       </c>
       <c r="D59">
-        <v>239.7913175011699</v>
+        <v>239.4550823770878</v>
       </c>
       <c r="E59">
-        <v>38.3714178384808</v>
+        <v>37.62969624391907</v>
       </c>
       <c r="F59">
-        <v>0.6450081759705886</v>
+        <v>0.6357036227313907</v>
       </c>
       <c r="G59">
-        <v>42.1783929270338</v>
+        <v>35</v>
       </c>
       <c r="H59">
-        <v>10570.04810597838</v>
+        <v>10576.06602859334</v>
       </c>
       <c r="I59">
-        <v>205.1340578278429</v>
+        <v>204.9586308270034</v>
       </c>
       <c r="J59">
-        <v>49.7922363954101</v>
+        <v>49.79245332653735</v>
       </c>
       <c r="K59">
-        <v>88.04855964395504</v>
+        <v>88.33574669077036</v>
       </c>
       <c r="L59">
-        <v>0.2221336808046557</v>
+        <v>0.2030562011648067</v>
       </c>
     </row>
     <row r="60" spans="1:12">
@@ -2676,34 +2676,34 @@
         <v>46327</v>
       </c>
       <c r="C60">
-        <v>59.8642701460678</v>
+        <v>59.01282835684326</v>
       </c>
       <c r="D60">
-        <v>239.4526351639035</v>
+        <v>239.7914524485976</v>
       </c>
       <c r="E60">
-        <v>38.50152274447638</v>
+        <v>37.35282770188717</v>
       </c>
       <c r="F60">
-        <v>0.6358456035346483</v>
+        <v>0.6260190020686751</v>
       </c>
       <c r="G60">
-        <v>41.75064137069001</v>
+        <v>35</v>
       </c>
       <c r="H60">
-        <v>10574.82338720954</v>
+        <v>10574.90532893854</v>
       </c>
       <c r="I60">
-        <v>205.0825767409012</v>
+        <v>205.1869710861339</v>
       </c>
       <c r="J60">
-        <v>49.79235945262307</v>
+        <v>49.79321116619966</v>
       </c>
       <c r="K60">
-        <v>88.32443849869163</v>
+        <v>88.35802364480573</v>
       </c>
       <c r="L60">
-        <v>0.2379785590462587</v>
+        <v>0.2061123419873219</v>
       </c>
     </row>
     <row r="61" spans="1:12">
@@ -2714,34 +2714,34 @@
         <v>46357</v>
       </c>
       <c r="C61">
-        <v>59.86164953994901</v>
+        <v>58.0162542184984</v>
       </c>
       <c r="D61">
-        <v>239.7929962041474</v>
+        <v>239.4558078406251</v>
       </c>
       <c r="E61">
-        <v>37.55996369534242</v>
+        <v>37.39756054214435</v>
       </c>
       <c r="F61">
-        <v>0.6432290013830302</v>
+        <v>0.6237782196394699</v>
       </c>
       <c r="G61">
-        <v>42.15000042426825</v>
+        <v>56.59358503005475</v>
       </c>
       <c r="H61">
-        <v>10574.6944035011</v>
+        <v>10571.97363168789</v>
       </c>
       <c r="I61">
-        <v>204.9296714119419</v>
+        <v>205.1705907123154</v>
       </c>
       <c r="J61">
-        <v>49.79269737416023</v>
+        <v>49.79200439297751</v>
       </c>
       <c r="K61">
-        <v>88.19714774257915</v>
+        <v>88.27375171430288</v>
       </c>
       <c r="L61">
-        <v>0.2206568578150738</v>
+        <v>0.2288555137728318</v>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -2752,34 +2752,34 @@
         <v>46388</v>
       </c>
       <c r="C62">
-        <v>59.94732467412157</v>
+        <v>52.97059197285058</v>
       </c>
       <c r="D62">
-        <v>239.452440819473</v>
+        <v>239.7918805491308</v>
       </c>
       <c r="E62">
-        <v>37.41964715802024</v>
+        <v>38.48298356806428</v>
       </c>
       <c r="F62">
-        <v>0.6280780944491247</v>
+        <v>0.6238763922612435</v>
       </c>
       <c r="G62">
-        <v>41.81668076108694</v>
+        <v>70.04939219470832</v>
       </c>
       <c r="H62">
-        <v>10570.08167339945</v>
+        <v>10574.46686248002</v>
       </c>
       <c r="I62">
-        <v>205.0348779522297</v>
+        <v>205.1679922037702</v>
       </c>
       <c r="J62">
-        <v>49.79226339407636</v>
+        <v>49.79272242335361</v>
       </c>
       <c r="K62">
-        <v>88.31262106678483</v>
+        <v>88.33761231032946</v>
       </c>
       <c r="L62">
-        <v>0.2318594210686706</v>
+        <v>0.2067132480703522</v>
       </c>
     </row>
     <row r="63" spans="1:12">
@@ -2790,34 +2790,34 @@
         <v>46419</v>
       </c>
       <c r="C63">
-        <v>59.94779393041308</v>
+        <v>51.30286009058332</v>
       </c>
       <c r="D63">
-        <v>239.4545434409765</v>
+        <v>239.789384225662</v>
       </c>
       <c r="E63">
-        <v>38.02302321359858</v>
+        <v>37.58994009556803</v>
       </c>
       <c r="F63">
-        <v>0.625414851497423</v>
+        <v>0.6317809172370477</v>
       </c>
       <c r="G63">
-        <v>41.64335561361196</v>
+        <v>53.28125826926858</v>
       </c>
       <c r="H63">
-        <v>10573.56433299276</v>
+        <v>10569.79666100302</v>
       </c>
       <c r="I63">
-        <v>205.2446900326868</v>
+        <v>205.2704152776659</v>
       </c>
       <c r="J63">
-        <v>49.79269732299305</v>
+        <v>49.79212242891008</v>
       </c>
       <c r="K63">
-        <v>88.29362530333748</v>
+        <v>88.32977462154977</v>
       </c>
       <c r="L63">
-        <v>0.2417308691147072</v>
+        <v>0.2327407960515176</v>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -2828,34 +2828,34 @@
         <v>46447</v>
       </c>
       <c r="C64">
-        <v>59.86319846225167</v>
+        <v>74.2625014913954</v>
       </c>
       <c r="D64">
-        <v>239.8057683607542</v>
+        <v>239.4517293301137</v>
       </c>
       <c r="E64">
-        <v>37.57583788738502</v>
+        <v>38.45038182256063</v>
       </c>
       <c r="F64">
-        <v>0.6273031951444903</v>
+        <v>0.629212062064344</v>
       </c>
       <c r="G64">
-        <v>42.90533199021016</v>
+        <v>38.91675903991105</v>
       </c>
       <c r="H64">
-        <v>10573.85642502113</v>
+        <v>10570.11400439204</v>
       </c>
       <c r="I64">
-        <v>205.0757886727457</v>
+        <v>205.1677438275399</v>
       </c>
       <c r="J64">
-        <v>49.79251088087054</v>
+        <v>49.79316909172634</v>
       </c>
       <c r="K64">
-        <v>88.12610209390256</v>
+        <v>88.35023181392825</v>
       </c>
       <c r="L64">
-        <v>0.2195545840224473</v>
+        <v>0.2185293646215248</v>
       </c>
     </row>
     <row r="65" spans="1:12">
@@ -2866,34 +2866,34 @@
         <v>46478</v>
       </c>
       <c r="C65">
-        <v>59.94550125151235</v>
+        <v>52.22572913985278</v>
       </c>
       <c r="D65">
-        <v>239.7971689879137</v>
+        <v>239.794671223146</v>
       </c>
       <c r="E65">
-        <v>38.15721877797465</v>
+        <v>38.2848125746617</v>
       </c>
       <c r="F65">
-        <v>0.6248343977293611</v>
+        <v>0.6250698398891074</v>
       </c>
       <c r="G65">
-        <v>42.5245375940757</v>
+        <v>44.14282740311371</v>
       </c>
       <c r="H65">
-        <v>10573.81408491862</v>
+        <v>10576.33115268902</v>
       </c>
       <c r="I65">
-        <v>205.1633795544268</v>
+        <v>205.1788991614537</v>
       </c>
       <c r="J65">
-        <v>49.79210159050854</v>
+        <v>49.79262958707839</v>
       </c>
       <c r="K65">
-        <v>88.28858522347795</v>
+        <v>88.23197295816587</v>
       </c>
       <c r="L65">
-        <v>0.2283041598958975</v>
+        <v>0.2173161514842511</v>
       </c>
     </row>
     <row r="66" spans="1:12">
@@ -2904,34 +2904,34 @@
         <v>46508</v>
       </c>
       <c r="C66">
-        <v>59.86411625368888</v>
+        <v>64.23716524802452</v>
       </c>
       <c r="D66">
-        <v>239.7949342351513</v>
+        <v>239.4489970018845</v>
       </c>
       <c r="E66">
-        <v>37.56942612736202</v>
+        <v>38.13983531273204</v>
       </c>
       <c r="F66">
-        <v>0.6259314104223958</v>
+        <v>0.6271328523020383</v>
       </c>
       <c r="G66">
-        <v>42.11685299677732</v>
+        <v>42.01457243310358</v>
       </c>
       <c r="H66">
-        <v>10570.8176400145</v>
+        <v>10570.08625101456</v>
       </c>
       <c r="I66">
-        <v>205.2223034610196</v>
+        <v>205.2046026894452</v>
       </c>
       <c r="J66">
-        <v>49.7928069453962</v>
+        <v>49.79216803951041</v>
       </c>
       <c r="K66">
-        <v>88.36881824258836</v>
+        <v>88.3762347458684</v>
       </c>
       <c r="L66">
-        <v>0.2130939169440687</v>
+        <v>0.2265653125245572</v>
       </c>
     </row>
     <row r="67" spans="1:12">
@@ -2942,34 +2942,34 @@
         <v>46539</v>
       </c>
       <c r="C67">
-        <v>59.8636828386853</v>
+        <v>58.8162468573488</v>
       </c>
       <c r="D67">
-        <v>239.8025590869516</v>
+        <v>239.802833822152</v>
       </c>
       <c r="E67">
-        <v>37.41964715802024</v>
+        <v>37.44244605806163</v>
       </c>
       <c r="F67">
-        <v>0.6277556697307641</v>
+        <v>0.6449762952059213</v>
       </c>
       <c r="G67">
-        <v>42.43712095955901</v>
+        <v>48.81649965029389</v>
       </c>
       <c r="H67">
-        <v>10574.35466764175</v>
+        <v>10576.39813466481</v>
       </c>
       <c r="I67">
-        <v>205.0742721673307</v>
+        <v>205.1788130545554</v>
       </c>
       <c r="J67">
-        <v>49.79272281490768</v>
+        <v>49.79239513222782</v>
       </c>
       <c r="K67">
-        <v>88.38939798451624</v>
+        <v>88.38467470297289</v>
       </c>
       <c r="L67">
-        <v>0.2346894397134751</v>
+        <v>0.2313227210473014</v>
       </c>
     </row>
     <row r="68" spans="1:12">
@@ -2980,34 +2980,34 @@
         <v>46569</v>
       </c>
       <c r="C68">
-        <v>59.86287878780269</v>
+        <v>64.99266752153011</v>
       </c>
       <c r="D68">
-        <v>239.759076583169</v>
+        <v>239.4522379936962</v>
       </c>
       <c r="E68">
-        <v>37.36876855347714</v>
+        <v>37.96294865703171</v>
       </c>
       <c r="F68">
-        <v>0.6337204330127661</v>
+        <v>0.6439679440144847</v>
       </c>
       <c r="G68">
-        <v>42.26258790756984</v>
+        <v>35</v>
       </c>
       <c r="H68">
-        <v>10570.39963020015</v>
+        <v>10576.07416149225</v>
       </c>
       <c r="I68">
-        <v>205.0770437506863</v>
+        <v>205.0956215392886</v>
       </c>
       <c r="J68">
-        <v>49.79245362261432</v>
+        <v>49.79260172773951</v>
       </c>
       <c r="K68">
-        <v>88.39055888478441</v>
+        <v>88.30703101553036</v>
       </c>
       <c r="L68">
-        <v>0.2151414360672533</v>
+        <v>0.2230854182955719</v>
       </c>
     </row>
     <row r="69" spans="1:12">
@@ -3018,34 +3018,34 @@
         <v>46600</v>
       </c>
       <c r="C69">
-        <v>59.86164953994901</v>
+        <v>61.28623960812671</v>
       </c>
       <c r="D69">
-        <v>239.455789894209</v>
+        <v>239.4538260136652</v>
       </c>
       <c r="E69">
-        <v>37.39865684630568</v>
+        <v>37.75094375565276</v>
       </c>
       <c r="F69">
-        <v>0.625747233058851</v>
+        <v>0.6290532906412371</v>
       </c>
       <c r="G69">
-        <v>42.54853414503638</v>
+        <v>38.71008988734938</v>
       </c>
       <c r="H69">
-        <v>10573.78534884698</v>
+        <v>10570.47754439223</v>
       </c>
       <c r="I69">
-        <v>205.2683905413865</v>
+        <v>204.9375719798004</v>
       </c>
       <c r="J69">
-        <v>49.79234351767096</v>
+        <v>49.79304958475407</v>
       </c>
       <c r="K69">
-        <v>88.32231028014164</v>
+        <v>88.10196822207247</v>
       </c>
       <c r="L69">
-        <v>0.2129835454005075</v>
+        <v>0.2187117858148574</v>
       </c>
     </row>
     <row r="70" spans="1:12">
@@ -3056,34 +3056,34 @@
         <v>46631</v>
       </c>
       <c r="C70">
-        <v>59.86254863503917</v>
+        <v>72.10605852004598</v>
       </c>
       <c r="D70">
-        <v>239.4488787224045</v>
+        <v>239.7820432663035</v>
       </c>
       <c r="E70">
-        <v>37.37644035813121</v>
+        <v>37.9321935606549</v>
       </c>
       <c r="F70">
-        <v>0.6245572503961159</v>
+        <v>0.6304837791684981</v>
       </c>
       <c r="G70">
-        <v>41.66305336683261</v>
+        <v>56.85658217780714</v>
       </c>
       <c r="H70">
-        <v>10573.91410411073</v>
+        <v>10570.02242666274</v>
       </c>
       <c r="I70">
-        <v>205.1559305464681</v>
+        <v>205.0968763771055</v>
       </c>
       <c r="J70">
-        <v>49.79295138151674</v>
+        <v>49.79302358910891</v>
       </c>
       <c r="K70">
-        <v>88.37997249554094</v>
+        <v>88.24827035041359</v>
       </c>
       <c r="L70">
-        <v>0.2069438124733851</v>
+        <v>0.2242683114043825</v>
       </c>
     </row>
     <row r="71" spans="1:12">
@@ -3094,34 +3094,34 @@
         <v>46661</v>
       </c>
       <c r="C71">
-        <v>59.95160957485869</v>
+        <v>66.02311638134987</v>
       </c>
       <c r="D71">
-        <v>239.4521287933179</v>
+        <v>239.7958891958554</v>
       </c>
       <c r="E71">
-        <v>37.53592985691783</v>
+        <v>37.39771939471287</v>
       </c>
       <c r="F71">
-        <v>0.6309785742218582</v>
+        <v>0.6360078256019651</v>
       </c>
       <c r="G71">
-        <v>41.64335561361196</v>
+        <v>40.47395491953031</v>
       </c>
       <c r="H71">
-        <v>10570.39963020015</v>
+        <v>10575.79843986021</v>
       </c>
       <c r="I71">
-        <v>204.9336873413791</v>
+        <v>205.0677690050489</v>
       </c>
       <c r="J71">
-        <v>49.79279197955242</v>
+        <v>49.79241564644387</v>
       </c>
       <c r="K71">
-        <v>88.41780246379358</v>
+        <v>88.37369180353065</v>
       </c>
       <c r="L71">
-        <v>0.2181813437805822</v>
+        <v>0.2179519436103501</v>
       </c>
     </row>
     <row r="72" spans="1:12">
@@ -3132,34 +3132,34 @@
         <v>46692</v>
       </c>
       <c r="C72">
-        <v>59.94794963253374</v>
+        <v>59.05933873213043</v>
       </c>
       <c r="D72">
-        <v>239.7945640504463</v>
+        <v>239.7948835187087</v>
       </c>
       <c r="E72">
-        <v>38.52126223237705</v>
+        <v>37.65036188876099</v>
       </c>
       <c r="F72">
-        <v>0.6306920729754381</v>
+        <v>0.6260821228637378</v>
       </c>
       <c r="G72">
-        <v>42.99877004150904</v>
+        <v>52.30083235064284</v>
       </c>
       <c r="H72">
-        <v>10573.42752623945</v>
+        <v>10574.61294770695</v>
       </c>
       <c r="I72">
-        <v>205.1033229291313</v>
+        <v>205.2596642091242</v>
       </c>
       <c r="J72">
-        <v>49.79203673463499</v>
+        <v>49.79290803429825</v>
       </c>
       <c r="K72">
-        <v>88.45193673982615</v>
+        <v>88.35379214680981</v>
       </c>
       <c r="L72">
-        <v>0.2185291197560923</v>
+        <v>0.2285198766113447</v>
       </c>
     </row>
     <row r="73" spans="1:12">
@@ -3170,34 +3170,34 @@
         <v>46722</v>
       </c>
       <c r="C73">
-        <v>59.86310395427682</v>
+        <v>75.45865027865742</v>
       </c>
       <c r="D73">
-        <v>239.4554820565302</v>
+        <v>239.7898240782054</v>
       </c>
       <c r="E73">
-        <v>37.60530995906422</v>
+        <v>37.59986125663824</v>
       </c>
       <c r="F73">
-        <v>0.6260353690732725</v>
+        <v>0.6258782855996242</v>
       </c>
       <c r="G73">
-        <v>41.9459341109058</v>
+        <v>62.69738954450903</v>
       </c>
       <c r="H73">
-        <v>10573.41548306681</v>
+        <v>10574.64707847283</v>
       </c>
       <c r="I73">
-        <v>205.0484556173944</v>
+        <v>205.1014382694822</v>
       </c>
       <c r="J73">
-        <v>49.79259280503816</v>
+        <v>49.79221204666078</v>
       </c>
       <c r="K73">
-        <v>87.99278703314745</v>
+        <v>88.07767095847856</v>
       </c>
       <c r="L73">
-        <v>0.226087364895831</v>
+        <v>0.2357170258810865</v>
       </c>
     </row>
     <row r="74" spans="1:12">
@@ -3208,34 +3208,34 @@
         <v>46023</v>
       </c>
       <c r="C74">
-        <v>56.79940873359313</v>
+        <v>58.43571608885521</v>
       </c>
       <c r="D74">
-        <v>227.2104802857598</v>
+        <v>227.1993073190567</v>
       </c>
       <c r="E74">
-        <v>35.52742420514767</v>
+        <v>35.50062938208531</v>
       </c>
       <c r="F74">
-        <v>0.6256909667892028</v>
+        <v>0.6258705717627054</v>
       </c>
       <c r="G74">
-        <v>42.39547208323274</v>
+        <v>51.88903663751851</v>
       </c>
       <c r="H74">
-        <v>10570.01567977228</v>
+        <v>10570.35046725442</v>
       </c>
       <c r="I74">
-        <v>194.5395418751488</v>
+        <v>194.4145027079911</v>
       </c>
       <c r="J74">
-        <v>49.79083909240398</v>
+        <v>49.79263059855538</v>
       </c>
       <c r="K74">
-        <v>85.82503004493248</v>
+        <v>85.93948950366671</v>
       </c>
       <c r="L74">
-        <v>0.1638536356429963</v>
+        <v>0.1928860855363207</v>
       </c>
     </row>
     <row r="75" spans="1:12">
@@ -3246,34 +3246,34 @@
         <v>46054</v>
       </c>
       <c r="C75">
-        <v>56.79936111014739</v>
+        <v>69.80151673872773</v>
       </c>
       <c r="D75">
-        <v>226.8784217001957</v>
+        <v>226.8859532414351</v>
       </c>
       <c r="E75">
-        <v>35.67762633848142</v>
+        <v>36.17582424066077</v>
       </c>
       <c r="F75">
-        <v>0.6245417062417544</v>
+        <v>0.6440495221646891</v>
       </c>
       <c r="G75">
-        <v>41.60252457265296</v>
+        <v>39.84789146720992</v>
       </c>
       <c r="H75">
-        <v>10573.25314603428</v>
+        <v>10571.41618494911</v>
       </c>
       <c r="I75">
-        <v>194.4585933224952</v>
+        <v>194.3873769198724</v>
       </c>
       <c r="J75">
-        <v>49.79071702232395</v>
+        <v>49.79219944081397</v>
       </c>
       <c r="K75">
-        <v>86.02112002251775</v>
+        <v>86.06464549891038</v>
       </c>
       <c r="L75">
-        <v>0.1777605009526583</v>
+        <v>0.1762432095413523</v>
       </c>
     </row>
     <row r="76" spans="1:12">
@@ -3284,34 +3284,34 @@
         <v>46082</v>
       </c>
       <c r="C76">
-        <v>56.79927809166382</v>
+        <v>58.00397369141447</v>
       </c>
       <c r="D76">
-        <v>226.8816384141253</v>
+        <v>227.2056501462957</v>
       </c>
       <c r="E76">
-        <v>35.48717596834742</v>
+        <v>35.46840783925536</v>
       </c>
       <c r="F76">
-        <v>0.6275353549526262</v>
+        <v>0.6276224396837481</v>
       </c>
       <c r="G76">
-        <v>42.24291067928134</v>
+        <v>46.6778073727854</v>
       </c>
       <c r="H76">
-        <v>10571.55289580747</v>
+        <v>10570.37395503224</v>
       </c>
       <c r="I76">
-        <v>194.2903907964595</v>
+        <v>194.3528056618019</v>
       </c>
       <c r="J76">
-        <v>49.79105577172051</v>
+        <v>49.79132529879037</v>
       </c>
       <c r="K76">
-        <v>85.97674637005436</v>
+        <v>85.97738566781692</v>
       </c>
       <c r="L76">
-        <v>0.1670674693019874</v>
+        <v>0.2008206173369463</v>
       </c>
     </row>
     <row r="77" spans="1:12">
@@ -3322,34 +3322,34 @@
         <v>46113</v>
       </c>
       <c r="C77">
-        <v>56.79653429491074</v>
+        <v>57.03084265449496</v>
       </c>
       <c r="D77">
-        <v>227.2065170380299</v>
+        <v>227.1959418082326</v>
       </c>
       <c r="E77">
-        <v>35.42155817897645</v>
+        <v>35.65419964131654</v>
       </c>
       <c r="F77">
-        <v>0.6276687047228573</v>
+        <v>0.6237820867753119</v>
       </c>
       <c r="G77">
-        <v>41.83069963242797</v>
+        <v>39.00858009987795</v>
       </c>
       <c r="H77">
-        <v>10569.55926115057</v>
+        <v>10571.18145562305</v>
       </c>
       <c r="I77">
-        <v>194.2878695980739</v>
+        <v>194.3498732001333</v>
       </c>
       <c r="J77">
-        <v>49.79092227141509</v>
+        <v>49.79232578642857</v>
       </c>
       <c r="K77">
-        <v>86.02061513338931</v>
+        <v>85.81533558494797</v>
       </c>
       <c r="L77">
-        <v>0.1784555379381587</v>
+        <v>0.1736077631965346</v>
       </c>
     </row>
     <row r="78" spans="1:12">
@@ -3360,34 +3360,34 @@
         <v>46143</v>
       </c>
       <c r="C78">
-        <v>56.71900939791499</v>
+        <v>55.16349107986543</v>
       </c>
       <c r="D78">
-        <v>227.1956596885524</v>
+        <v>227.2020269977902</v>
       </c>
       <c r="E78">
-        <v>36.38110851292772</v>
+        <v>36.536197772528</v>
       </c>
       <c r="F78">
-        <v>0.6428929535316134</v>
+        <v>0.6303825516912752</v>
       </c>
       <c r="G78">
-        <v>41.82408599230251</v>
+        <v>35</v>
       </c>
       <c r="H78">
-        <v>10575.86944004957</v>
+        <v>10575.8623386498</v>
       </c>
       <c r="I78">
-        <v>194.4193961107665</v>
+        <v>194.4362959208648</v>
       </c>
       <c r="J78">
-        <v>49.79112890693455</v>
+        <v>49.79320243273575</v>
       </c>
       <c r="K78">
-        <v>85.95218252688569</v>
+        <v>85.94195667327176</v>
       </c>
       <c r="L78">
-        <v>0.1717851800939136</v>
+        <v>0.2040407423227836</v>
       </c>
     </row>
     <row r="79" spans="1:12">
@@ -3398,34 +3398,34 @@
         <v>46174</v>
       </c>
       <c r="C79">
-        <v>56.71952451090148</v>
+        <v>56.94454639127272</v>
       </c>
       <c r="D79">
-        <v>227.2104802857598</v>
+        <v>227.1978315534693</v>
       </c>
       <c r="E79">
-        <v>36.28648203478411</v>
+        <v>35.54808264130674</v>
       </c>
       <c r="F79">
-        <v>0.6284150798212286</v>
+        <v>0.6346167541414712</v>
       </c>
       <c r="G79">
-        <v>41.7431097298541</v>
+        <v>48.59657418040548</v>
       </c>
       <c r="H79">
-        <v>10570.17360991625</v>
+        <v>10574.22151363082</v>
       </c>
       <c r="I79">
-        <v>194.4274885933322</v>
+        <v>194.3338824669007</v>
       </c>
       <c r="J79">
-        <v>49.79326359118424</v>
+        <v>49.79234751274107</v>
       </c>
       <c r="K79">
-        <v>85.98824215574935</v>
+        <v>85.95911506521779</v>
       </c>
       <c r="L79">
-        <v>0.2207631750870736</v>
+        <v>0.2166327596591025</v>
       </c>
     </row>
     <row r="80" spans="1:12">
@@ -3436,34 +3436,34 @@
         <v>46204</v>
       </c>
       <c r="C80">
-        <v>56.80252703145352</v>
+        <v>55.43840294272168</v>
       </c>
       <c r="D80">
-        <v>226.8758453394154</v>
+        <v>226.8867698437791</v>
       </c>
       <c r="E80">
-        <v>35.85207506322565</v>
+        <v>35.85178481398719</v>
       </c>
       <c r="F80">
-        <v>0.6245417062417544</v>
+        <v>0.6461574815832285</v>
       </c>
       <c r="G80">
-        <v>41.80214608648519</v>
+        <v>35.59049493835047</v>
       </c>
       <c r="H80">
-        <v>10575.66641788145</v>
+        <v>10571.51485870137</v>
       </c>
       <c r="I80">
-        <v>194.4944117754793</v>
+        <v>194.4433876122924</v>
       </c>
       <c r="J80">
-        <v>49.79312511210506</v>
+        <v>49.79215896823683</v>
       </c>
       <c r="K80">
-        <v>85.97911949055283</v>
+        <v>85.89674173526679</v>
       </c>
       <c r="L80">
-        <v>0.2209130534109502</v>
+        <v>0.2295531558361632</v>
       </c>
     </row>
     <row r="81" spans="1:12">
@@ -3474,34 +3474,34 @@
         <v>46235</v>
       </c>
       <c r="C81">
-        <v>56.7185560308476</v>
+        <v>53.50865532721667</v>
       </c>
       <c r="D81">
-        <v>227.1968257138978</v>
+        <v>226.8824638629779</v>
       </c>
       <c r="E81">
-        <v>35.4075192726443</v>
+        <v>35.54554359350784</v>
       </c>
       <c r="F81">
-        <v>0.6342076337594031</v>
+        <v>0.6302934710973006</v>
       </c>
       <c r="G81">
-        <v>41.90103948353364</v>
+        <v>42.99948440576091</v>
       </c>
       <c r="H81">
-        <v>10575.22000450655</v>
+        <v>10569.93020479541</v>
       </c>
       <c r="I81">
-        <v>194.4224137536252</v>
+        <v>194.5225435061529</v>
       </c>
       <c r="J81">
-        <v>49.79030973176612</v>
+        <v>49.793120863985</v>
       </c>
       <c r="K81">
-        <v>85.89839676159896</v>
+        <v>85.86895298559635</v>
       </c>
       <c r="L81">
-        <v>0.1788223912194385</v>
+        <v>0.2075031651134517</v>
       </c>
     </row>
     <row r="82" spans="1:12">
@@ -3512,34 +3512,34 @@
         <v>46266</v>
       </c>
       <c r="C82">
-        <v>56.71964846922576</v>
+        <v>56.46422103205033</v>
       </c>
       <c r="D82">
-        <v>226.8804135603216</v>
+        <v>226.8888715427055</v>
       </c>
       <c r="E82">
-        <v>35.70000101007944</v>
+        <v>36.71848235112656</v>
       </c>
       <c r="F82">
-        <v>0.6319978501454784</v>
+        <v>0.6347483416575185</v>
       </c>
       <c r="G82">
-        <v>41.70855862248433</v>
+        <v>38.4936242358372</v>
       </c>
       <c r="H82">
-        <v>10571.86188270665</v>
+        <v>10576.05963534609</v>
       </c>
       <c r="I82">
-        <v>194.4275965737172</v>
+        <v>194.5159229194242</v>
       </c>
       <c r="J82">
-        <v>49.79131181770563</v>
+        <v>49.79288857453187</v>
       </c>
       <c r="K82">
-        <v>86.04334846996342</v>
+        <v>85.93062053166823</v>
       </c>
       <c r="L82">
-        <v>0.2050698746099258</v>
+        <v>0.1968339720265526</v>
       </c>
     </row>
     <row r="83" spans="1:12">
@@ -3550,34 +3550,34 @@
         <v>46296</v>
       </c>
       <c r="C83">
-        <v>56.71987893085225</v>
+        <v>60.66923194634959</v>
       </c>
       <c r="D83">
-        <v>227.200075953745</v>
+        <v>227.188264837296</v>
       </c>
       <c r="E83">
-        <v>35.6527426775798</v>
+        <v>36.06828201235569</v>
       </c>
       <c r="F83">
-        <v>0.6281547149923287</v>
+        <v>0.6267635658116023</v>
       </c>
       <c r="G83">
-        <v>42.22843407025439</v>
+        <v>43.42655280141894</v>
       </c>
       <c r="H83">
-        <v>10575.33196719844</v>
+        <v>10576.03184633758</v>
       </c>
       <c r="I83">
-        <v>194.3990423781397</v>
+        <v>194.4196111224004</v>
       </c>
       <c r="J83">
-        <v>49.79156047984267</v>
+        <v>49.79264145179143</v>
       </c>
       <c r="K83">
-        <v>85.77735320028289</v>
+        <v>85.94798251993168</v>
       </c>
       <c r="L83">
-        <v>0.1784031438476152</v>
+        <v>0.1936035002596352</v>
       </c>
     </row>
     <row r="84" spans="1:12">
@@ -3588,34 +3588,34 @@
         <v>46327</v>
       </c>
       <c r="C84">
-        <v>56.71887106813924</v>
+        <v>53.41299277169325</v>
       </c>
       <c r="D84">
-        <v>227.1835373276831</v>
+        <v>226.8912140872051</v>
       </c>
       <c r="E84">
-        <v>35.54990620542725</v>
+        <v>36.66224550405796</v>
       </c>
       <c r="F84">
-        <v>0.6265327448716035</v>
+        <v>0.6237820867753119</v>
       </c>
       <c r="G84">
-        <v>41.61733713296773</v>
+        <v>57.39788688545527</v>
       </c>
       <c r="H84">
-        <v>10574.21139801236</v>
+        <v>10575.58710969068</v>
       </c>
       <c r="I84">
-        <v>194.44020259685</v>
+        <v>194.2874597050902</v>
       </c>
       <c r="J84">
-        <v>49.79081602179562</v>
+        <v>49.79215840796834</v>
       </c>
       <c r="K84">
-        <v>85.81645723982747</v>
+        <v>86.02232423750559</v>
       </c>
       <c r="L84">
-        <v>0.1996762481466046</v>
+        <v>0.1705704181689208</v>
       </c>
     </row>
     <row r="85" spans="1:12">
@@ -3626,34 +3626,34 @@
         <v>46357</v>
       </c>
       <c r="C85">
-        <v>56.71825607053818</v>
+        <v>71.98178324726408</v>
       </c>
       <c r="D85">
-        <v>227.200805825424</v>
+        <v>227.1996093913978</v>
       </c>
       <c r="E85">
-        <v>36.05116814046262</v>
+        <v>35.59519947116043</v>
       </c>
       <c r="F85">
-        <v>0.6246798178913735</v>
+        <v>0.6282771278397055</v>
       </c>
       <c r="G85">
-        <v>43.14381974768909</v>
+        <v>45.24399130078043</v>
       </c>
       <c r="H85">
-        <v>10575.40768820473</v>
+        <v>10573.817381339</v>
       </c>
       <c r="I85">
-        <v>194.4215803934979</v>
+        <v>194.4168792594825</v>
       </c>
       <c r="J85">
-        <v>49.79068444622074</v>
+        <v>49.79278066230992</v>
       </c>
       <c r="K85">
-        <v>86.00111002122739</v>
+        <v>85.93215720409187</v>
       </c>
       <c r="L85">
-        <v>0.219606108454068</v>
+        <v>0.2022713917455778</v>
       </c>
     </row>
     <row r="86" spans="1:12">
@@ -3664,34 +3664,34 @@
         <v>46388</v>
       </c>
       <c r="C86">
-        <v>56.79922540955083</v>
+        <v>53.82865268947327</v>
       </c>
       <c r="D86">
-        <v>226.880749963701</v>
+        <v>227.1993073190567</v>
       </c>
       <c r="E86">
-        <v>35.46794446980947</v>
+        <v>36.13729309508952</v>
       </c>
       <c r="F86">
-        <v>0.6395078548519204</v>
+        <v>0.6363649264950101</v>
       </c>
       <c r="G86">
-        <v>42.42649545112861</v>
+        <v>35</v>
       </c>
       <c r="H86">
-        <v>10574.94977400352</v>
+        <v>10571.41274995597</v>
       </c>
       <c r="I86">
-        <v>194.3929322347139</v>
+        <v>194.4124509688134</v>
       </c>
       <c r="J86">
-        <v>49.79042410856771</v>
+        <v>49.79191708238854</v>
       </c>
       <c r="K86">
-        <v>86.03549798939729</v>
+        <v>86.02838958591039</v>
       </c>
       <c r="L86">
-        <v>0.1736414956617103</v>
+        <v>0.1765330609896727</v>
       </c>
     </row>
     <row r="87" spans="1:12">
@@ -3702,34 +3702,34 @@
         <v>46419</v>
       </c>
       <c r="C87">
-        <v>56.79969284819278</v>
+        <v>56.27583848591001</v>
       </c>
       <c r="D87">
-        <v>226.8834315318306</v>
+        <v>227.2060928050834</v>
       </c>
       <c r="E87">
-        <v>35.72880983151772</v>
+        <v>36.9623641248733</v>
       </c>
       <c r="F87">
-        <v>0.6317607590980354</v>
+        <v>0.6242050550544994</v>
       </c>
       <c r="G87">
-        <v>41.75678189177645</v>
+        <v>44.87860968868836</v>
       </c>
       <c r="H87">
-        <v>10570.38417370513</v>
+        <v>10573.74718650638</v>
       </c>
       <c r="I87">
-        <v>194.5046656790069</v>
+        <v>194.4118386739711</v>
       </c>
       <c r="J87">
-        <v>49.79123460616527</v>
+        <v>49.7919574997003</v>
       </c>
       <c r="K87">
-        <v>85.96955826152204</v>
+        <v>86.0180820615624</v>
       </c>
       <c r="L87">
-        <v>0.2145800697620015</v>
+        <v>0.2239855171461046</v>
       </c>
     </row>
     <row r="88" spans="1:12">
@@ -3740,34 +3740,34 @@
         <v>46447</v>
       </c>
       <c r="C88">
-        <v>56.71851280328694</v>
+        <v>49.93840620710751</v>
       </c>
       <c r="D88">
-        <v>226.87243269228</v>
+        <v>226.8929289169826</v>
       </c>
       <c r="E88">
-        <v>35.5624430578298</v>
+        <v>36.32487889685149</v>
       </c>
       <c r="F88">
-        <v>0.6247919941258017</v>
+        <v>0.6249578092202079</v>
       </c>
       <c r="G88">
-        <v>41.83095725397136</v>
+        <v>41.5349160646606</v>
       </c>
       <c r="H88">
-        <v>10573.51886354721</v>
+        <v>10571.40471880405</v>
       </c>
       <c r="I88">
-        <v>194.1972376846168</v>
+        <v>194.4481167586916</v>
       </c>
       <c r="J88">
-        <v>49.79084243125322</v>
+        <v>49.79185165281147</v>
       </c>
       <c r="K88">
-        <v>85.90918431995937</v>
+        <v>85.97558157182031</v>
       </c>
       <c r="L88">
-        <v>0.1861963974170253</v>
+        <v>0.1768113474962913</v>
       </c>
     </row>
     <row r="89" spans="1:12">
@@ -3778,34 +3778,34 @@
         <v>46478</v>
       </c>
       <c r="C89">
-        <v>56.71797586006409</v>
+        <v>56.54860688565647</v>
       </c>
       <c r="D89">
-        <v>227.1958773148703</v>
+        <v>226.8799929569227</v>
       </c>
       <c r="E89">
-        <v>35.42788902585201</v>
+        <v>35.5332511206893</v>
       </c>
       <c r="F89">
-        <v>0.6278493748311402</v>
+        <v>0.6414359993801757</v>
       </c>
       <c r="G89">
-        <v>42.68668843475559</v>
+        <v>59.98415936401311</v>
       </c>
       <c r="H89">
-        <v>10574.17381344301</v>
+        <v>10570.55653571093</v>
       </c>
       <c r="I89">
-        <v>194.401876512478</v>
+        <v>194.3643747465238</v>
       </c>
       <c r="J89">
-        <v>49.79199960880177</v>
+        <v>49.79275889290705</v>
       </c>
       <c r="K89">
-        <v>86.00803674252857</v>
+        <v>85.98431483949534</v>
       </c>
       <c r="L89">
-        <v>0.2111769295636055</v>
+        <v>0.2230977913492065</v>
       </c>
     </row>
     <row r="90" spans="1:12">
@@ -3816,34 +3816,34 @@
         <v>46508</v>
       </c>
       <c r="C90">
-        <v>56.71870553285193</v>
+        <v>55.07479371882934</v>
       </c>
       <c r="D90">
-        <v>227.2000991900223</v>
+        <v>227.19636501403</v>
       </c>
       <c r="E90">
-        <v>35.82870360422638</v>
+        <v>36.70371086367695</v>
       </c>
       <c r="F90">
-        <v>0.6286946256648018</v>
+        <v>0.6242879058323593</v>
       </c>
       <c r="G90">
-        <v>43.05310601320825</v>
+        <v>35</v>
       </c>
       <c r="H90">
-        <v>10573.85105084869</v>
+        <v>10571.52563575583</v>
       </c>
       <c r="I90">
-        <v>194.4456035554426</v>
+        <v>194.3940258337875</v>
       </c>
       <c r="J90">
-        <v>49.79129269333958</v>
+        <v>49.79274506863364</v>
       </c>
       <c r="K90">
-        <v>85.95575876156096</v>
+        <v>86.0451454252748</v>
       </c>
       <c r="L90">
-        <v>0.2064512936116937</v>
+        <v>0.1909613148342666</v>
       </c>
     </row>
     <row r="91" spans="1:12">
@@ -3854,34 +3854,34 @@
         <v>46539</v>
       </c>
       <c r="C91">
-        <v>56.71843632851736</v>
+        <v>51.37320132781007</v>
       </c>
       <c r="D91">
-        <v>226.8752105559546</v>
+        <v>227.1592617635541</v>
       </c>
       <c r="E91">
-        <v>36.73545799025909</v>
+        <v>35.40884760857737</v>
       </c>
       <c r="F91">
-        <v>0.6244802565847544</v>
+        <v>0.643833629943266</v>
       </c>
       <c r="G91">
-        <v>43.08327674259906</v>
+        <v>40.15860453295516</v>
       </c>
       <c r="H91">
-        <v>10573.78509706901</v>
+        <v>10574.24662565297</v>
       </c>
       <c r="I91">
-        <v>194.4336631628059</v>
+        <v>194.448617392553</v>
       </c>
       <c r="J91">
-        <v>49.79045763903842</v>
+        <v>49.79260697163932</v>
       </c>
       <c r="K91">
-        <v>85.99151612233986</v>
+        <v>86.01057948309422</v>
       </c>
       <c r="L91">
-        <v>0.2264184413935528</v>
+        <v>0.2208780791789162</v>
       </c>
     </row>
     <row r="92" spans="1:12">
@@ -3892,34 +3892,34 @@
         <v>46569</v>
       </c>
       <c r="C92">
-        <v>56.71900939791499</v>
+        <v>62.95759869920136</v>
       </c>
       <c r="D92">
-        <v>226.8747053964066</v>
+        <v>227.181473439744</v>
       </c>
       <c r="E92">
-        <v>35.5111985093369</v>
+        <v>36.68426818213477</v>
       </c>
       <c r="F92">
-        <v>0.6259799828206293</v>
+        <v>0.6286283398106806</v>
       </c>
       <c r="G92">
-        <v>42.02305142583165</v>
+        <v>41.01508385257032</v>
       </c>
       <c r="H92">
-        <v>10571.74336535642</v>
+        <v>10576.07077580843</v>
       </c>
       <c r="I92">
-        <v>194.4579606195674</v>
+        <v>194.3511084625278</v>
       </c>
       <c r="J92">
-        <v>49.79188411932775</v>
+        <v>49.7925065353695</v>
       </c>
       <c r="K92">
-        <v>85.99883334321078</v>
+        <v>85.86699124979181</v>
       </c>
       <c r="L92">
-        <v>0.1595627442408799</v>
+        <v>0.1943834531723632</v>
       </c>
     </row>
     <row r="93" spans="1:12">
@@ -3930,34 +3930,34 @@
         <v>46600</v>
       </c>
       <c r="C93">
-        <v>56.71937776268724</v>
+        <v>76.40082781509643</v>
       </c>
       <c r="D93">
-        <v>227.2007845018088</v>
+        <v>227.1976371634287</v>
       </c>
       <c r="E93">
-        <v>35.56897108467118</v>
+        <v>35.76568218231314</v>
       </c>
       <c r="F93">
-        <v>0.6339958161882923</v>
+        <v>0.6252708375725733</v>
       </c>
       <c r="G93">
-        <v>42.01362631049812</v>
+        <v>50.21829807848817</v>
       </c>
       <c r="H93">
-        <v>10573.53114808842</v>
+        <v>10576.36600607178</v>
       </c>
       <c r="I93">
-        <v>194.3217903595762</v>
+        <v>194.1838462191761</v>
       </c>
       <c r="J93">
-        <v>49.7904614631709</v>
+        <v>49.79193751669403</v>
       </c>
       <c r="K93">
-        <v>86.011807347032</v>
+        <v>85.94169151512779</v>
       </c>
       <c r="L93">
-        <v>0.1732250252609482</v>
+        <v>0.197165023543961</v>
       </c>
     </row>
     <row r="94" spans="1:12">
@@ -3968,34 +3968,34 @@
         <v>46631</v>
       </c>
       <c r="C94">
-        <v>56.80237002026787</v>
+        <v>59.43113736506287</v>
       </c>
       <c r="D94">
-        <v>227.200805825424</v>
+        <v>227.1993073190567</v>
       </c>
       <c r="E94">
-        <v>35.67641156731313</v>
+        <v>35.47190991513749</v>
       </c>
       <c r="F94">
-        <v>0.6276452348622487</v>
+        <v>0.6263475454824016</v>
       </c>
       <c r="G94">
-        <v>42.71900698233281</v>
+        <v>35</v>
       </c>
       <c r="H94">
-        <v>10575.33196719844</v>
+        <v>10575.97259022902</v>
       </c>
       <c r="I94">
-        <v>194.2119767981461</v>
+        <v>194.415081762119</v>
       </c>
       <c r="J94">
-        <v>49.79041721781483</v>
+        <v>49.79264117194873</v>
       </c>
       <c r="K94">
-        <v>85.9829185855269</v>
+        <v>85.99475674413942</v>
       </c>
       <c r="L94">
-        <v>0.1867585091727951</v>
+        <v>0.222644950683551</v>
       </c>
     </row>
     <row r="95" spans="1:12">
@@ -4006,34 +4006,34 @@
         <v>46661</v>
       </c>
       <c r="C95">
-        <v>56.79632776766795</v>
+        <v>57.01476116862779</v>
       </c>
       <c r="D95">
-        <v>227.1969968676612</v>
+        <v>227.2103315407264</v>
       </c>
       <c r="E95">
-        <v>35.51474858431333</v>
+        <v>35.67653549348446</v>
       </c>
       <c r="F95">
-        <v>0.6289132588434905</v>
+        <v>0.6259644375846779</v>
       </c>
       <c r="G95">
-        <v>41.70123497005871</v>
+        <v>54.57550722064541</v>
       </c>
       <c r="H95">
-        <v>10571.65055704174</v>
+        <v>10575.75633883007</v>
       </c>
       <c r="I95">
-        <v>194.4511701401518</v>
+        <v>194.4051099938966</v>
       </c>
       <c r="J95">
-        <v>49.79120730548467</v>
+        <v>49.79228770592967</v>
       </c>
       <c r="K95">
-        <v>85.97189819682663</v>
+        <v>85.9513096908439</v>
       </c>
       <c r="L95">
-        <v>0.1728599284797962</v>
+        <v>0.194153125911163</v>
       </c>
     </row>
     <row r="96" spans="1:12">
@@ -4044,34 +4044,34 @@
         <v>46692</v>
       </c>
       <c r="C96">
-        <v>56.71865121316023</v>
+        <v>54.64469837032016</v>
       </c>
       <c r="D96">
-        <v>227.2107644385637</v>
+        <v>227.2059437483844</v>
       </c>
       <c r="E96">
-        <v>35.4682059339876</v>
+        <v>35.97318539873175</v>
       </c>
       <c r="F96">
-        <v>0.632892036638049</v>
+        <v>0.6285557369506526</v>
       </c>
       <c r="G96">
-        <v>43.08928989390233</v>
+        <v>36.66236046729216</v>
       </c>
       <c r="H96">
-        <v>10575.19916774601</v>
+        <v>10571.37083665696</v>
       </c>
       <c r="I96">
-        <v>194.3118401156436</v>
+        <v>194.425164315702</v>
       </c>
       <c r="J96">
-        <v>49.79120962708548</v>
+        <v>49.79305669348511</v>
       </c>
       <c r="K96">
-        <v>86.01909272214128</v>
+        <v>86.01899103629745</v>
       </c>
       <c r="L96">
-        <v>0.2067192788905761</v>
+        <v>0.1768537842024297</v>
       </c>
     </row>
     <row r="97" spans="1:12">
@@ -4082,34 +4082,34 @@
         <v>46722</v>
       </c>
       <c r="C97">
-        <v>56.79940292452382</v>
+        <v>54.40258831675103</v>
       </c>
       <c r="D97">
-        <v>227.1847602028178</v>
+        <v>226.8847979941497</v>
       </c>
       <c r="E97">
-        <v>35.73508749641852</v>
+        <v>35.46352277474023</v>
       </c>
       <c r="F97">
-        <v>0.6257323175425767</v>
+        <v>0.6357863999782084</v>
       </c>
       <c r="G97">
-        <v>41.79962717639577</v>
+        <v>38.49224382501621</v>
       </c>
       <c r="H97">
-        <v>10571.79647947195</v>
+        <v>10575.91526109631</v>
       </c>
       <c r="I97">
-        <v>194.3121161874367</v>
+        <v>194.3309511033</v>
       </c>
       <c r="J97">
-        <v>49.79038279065995</v>
+        <v>49.79195555213526</v>
       </c>
       <c r="K97">
-        <v>85.99590159265435</v>
+        <v>85.95686850292735</v>
       </c>
       <c r="L97">
-        <v>0.2153277378895595</v>
+        <v>0.2167509645113485</v>
       </c>
     </row>
   </sheetData>

</xml_diff>